<commit_message>
Rett navn og oppdater publiserte resultater
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -660,7 +660,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Bj?rnar Slettv?g</t>
+          <t>Bjørnar Slettvåg</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Alva Witnes Ertresv?g</t>
+          <t>Alva Witnes Ertresvåg</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Rett Kristian Frøyen i publiserte resultater
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -579,7 +579,7 @@
         <v>381</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>44</v>
@@ -1028,7 +1028,11 @@
           <t>17</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>Klassevinner. Beste kvinne totalt</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1188,7 +1192,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Kristian Fr?yen</t>
+          <t>Kristian Frøyen</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Fix Norwegian character encoding
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -670,7 +670,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>K ?pen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -958,7 +958,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>K ?pen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1006,7 +1006,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1194,7 +1194,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>M ?pen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Fix Norwegian characters in event names
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -1271,7 +1271,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Oslo L?psfestival - 5'ern v?r!</t>
+          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Oslo L?psfestival - 5'ern v?r!</t>
+          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Oslo L?psfestival - 5'ern v?r!</t>
+          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Oslo L?psfestival - 5'ern v?r!</t>
+          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Oslo L?psfestival - 5'ern v?r!</t>
+          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Oslo L?psfestival - 5'ern v?r!</t>
+          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Oslo L?psfestival - 5'ern v?r!</t>
+          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>NM terrengl?p kort l?ype</t>
+          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>NM terrengl?p kort l?ype</t>
+          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -1879,7 +1879,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>NM terrengl?p kort l?ype</t>
+          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>NM terrengl?p kort l?ype</t>
+          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>NM terrengl?p kort l?ype</t>
+          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>K ?pen</t>
+          <t>K Ã¥pen</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
@@ -20671,7 +20671,7 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>3000 St. Haugen og Salomon, Bislett distanseserie 4- 3K, Leipzig Marathon, NM terrengl?p kort l?ype, Oslo L?psfestival - 5'ern v?r!, Perseløpet #1 - 2026, Seven Hills Record Run, Österlen Spring Trail Duo Trail</t>
+          <t>3000 St. Haugen og Salomon, Bislett distanseserie 4- 3K, Leipzig Marathon, NM terrenglÃ¸p kort lÃ¸ype, Oslo LÃ¸psfestival - 5'ern vÃ¥r!, Perseløpet #1 - 2026, Seven Hills Record Run, Österlen Spring Trail Duo Trail</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix mojibake in published results
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -579,7 +579,7 @@
         <v>429</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>53</v>
@@ -1271,7 +1271,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
+          <t>Oslo Løpsfestival - 5'ern vår!</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
+          <t>Oslo Løpsfestival - 5'ern vår!</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
+          <t>Oslo Løpsfestival - 5'ern vår!</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
+          <t>Oslo Løpsfestival - 5'ern vår!</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
+          <t>Oslo Løpsfestival - 5'ern vår!</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1523,7 +1523,7 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
+          <t>Oslo Løpsfestival - 5'ern vår!</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Oslo LÃ¸psfestival - 5'ern vÃ¥r!</t>
+          <t>Oslo Løpsfestival - 5'ern vår!</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>Anna Marie SirevÃ¥g</t>
+          <t>Anna Marie Sirevåg</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
@@ -1932,8 +1932,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Ã-dne Andersen Andersen</t>
+          <t>Ådne Andersen Andersen</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -1981,7 +1980,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>MadelÃ¨ne Holum</t>
+          <t>Madelène Holum</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -2024,7 +2023,7 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
+          <t>NM terrengløp kort løype</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -2072,7 +2071,7 @@
       </c>
       <c r="C38" s="7" t="inlineStr">
         <is>
-          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
+          <t>NM terrengløp kort løype</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -2120,7 +2119,7 @@
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
+          <t>NM terrengløp kort løype</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -2168,7 +2167,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
+          <t>NM terrengløp kort løype</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -2216,7 +2215,7 @@
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>NM terrenglÃ¸p kort lÃ¸ype</t>
+          <t>NM terrengløp kort løype</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -2279,7 +2278,7 @@
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>K Ã¥pen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Deduplicate athlete names in rankings
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -579,7 +579,7 @@
         <v>429</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>53</v>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>Madelène Holum</t>
+          <t>Madelène Wanvik Holum</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update Anna Marie Sirevåg name
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -579,7 +579,7 @@
         <v>429</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>53</v>
@@ -16772,7 +16772,7 @@
       </c>
       <c r="D349" s="7" t="inlineStr">
         <is>
-          <t>anna sir</t>
+          <t>Anna Marie Sirevåg</t>
         </is>
       </c>
       <c r="E349" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Fix Sentrumsløpet gender assignments
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -1241,7 +1241,7 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1433,7 +1433,7 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1481,7 +1481,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -2345,7 +2345,7 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -2537,7 +2537,7 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F54" s="6" t="inlineStr">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F62" s="6" t="inlineStr">
@@ -3257,7 +3257,7 @@
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
@@ -3401,7 +3401,7 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F68" s="6" t="inlineStr">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
@@ -3593,7 +3593,7 @@
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
@@ -3689,7 +3689,7 @@
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="E74" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
@@ -3837,7 +3837,7 @@
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F80" s="6" t="inlineStr">
@@ -4125,7 +4125,7 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
@@ -4317,7 +4317,7 @@
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
@@ -4797,7 +4797,7 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
@@ -4845,7 +4845,7 @@
       </c>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="E98" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F98" s="6" t="inlineStr">
@@ -5277,7 +5277,7 @@
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F106" s="6" t="inlineStr">
@@ -5469,7 +5469,7 @@
       </c>
       <c r="E109" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F109" s="6" t="inlineStr">
@@ -5661,7 +5661,7 @@
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="E125" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F125" s="6" t="inlineStr">
@@ -6289,7 +6289,7 @@
       </c>
       <c r="E126" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F126" s="6" t="inlineStr">
@@ -6389,7 +6389,7 @@
       </c>
       <c r="E128" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F128" s="6" t="inlineStr">
@@ -6629,7 +6629,7 @@
       </c>
       <c r="E133" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F133" s="6" t="inlineStr">
@@ -6677,7 +6677,7 @@
       </c>
       <c r="E134" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F134" s="6" t="inlineStr">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="E135" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F135" s="6" t="inlineStr">
@@ -6773,7 +6773,7 @@
       </c>
       <c r="E136" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F136" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update Grue pacer note
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -1024,7 +1024,11 @@
           <t>182</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update Sundvolden hill race note
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -2360,7 +2360,11 @@
           <t>2</t>
         </is>
       </c>
-      <c r="J43" s="7" t="inlineStr"/>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>motbakkeløp</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update Revetal class placements
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -2906,7 +2906,7 @@
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>K35-39</t>
+          <t>K23-39</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>K23-34</t>
+          <t>K23-39</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>M23-34</t>
+          <t>M23-39</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Merk fartsholdere i Sommernattslopet
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -7020,7 +7020,11 @@
           <t>35</t>
         </is>
       </c>
-      <c r="J134" s="7" t="inlineStr"/>
+      <c r="J134" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
@@ -7214,7 +7218,7 @@
       </c>
       <c r="J138" s="7" t="inlineStr">
         <is>
-          <t>relatert treff</t>
+          <t>fartsholder</t>
         </is>
       </c>
     </row>
@@ -7552,7 +7556,11 @@
           <t>53</t>
         </is>
       </c>
-      <c r="J145" s="7" t="inlineStr"/>
+      <c r="J145" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="6" t="inlineStr">
@@ -7700,7 +7708,11 @@
           <t>61</t>
         </is>
       </c>
-      <c r="J148" s="7" t="inlineStr"/>
+      <c r="J148" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Merk Simon 10 km som fartsholder
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -7508,7 +7508,11 @@
           <t>237</t>
         </is>
       </c>
-      <c r="J144" s="7" t="inlineStr"/>
+      <c r="J144" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Beregn flere WA-poeng for standarddistanser
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -9616,7 +9616,7 @@
       </c>
       <c r="D187" s="7" t="inlineStr">
         <is>
-          <t>Anna Marie Nordengen Sirevåg</t>
+          <t>Vilde Våge Henriksen</t>
         </is>
       </c>
       <c r="E187" s="6" t="inlineStr">
@@ -9631,22 +9631,22 @@
       </c>
       <c r="G187" s="6" t="inlineStr">
         <is>
-          <t>5000 m</t>
+          <t>3000 m hinder</t>
         </is>
       </c>
       <c r="H187" s="7" t="inlineStr">
         <is>
-          <t>15:23.39</t>
+          <t>9:40.58</t>
         </is>
       </c>
       <c r="I187" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>3</t>
         </is>
       </c>
       <c r="J187" s="7" t="inlineStr">
         <is>
-          <t>PB, norsk U23-rekord</t>
+          <t>PB</t>
         </is>
       </c>
     </row>
@@ -9668,7 +9668,7 @@
       </c>
       <c r="D188" s="7" t="inlineStr">
         <is>
-          <t>Vilde Våge Henriksen</t>
+          <t>Anna Marie Nordengen Sirevåg</t>
         </is>
       </c>
       <c r="E188" s="6" t="inlineStr">
@@ -9683,22 +9683,22 @@
       </c>
       <c r="G188" s="6" t="inlineStr">
         <is>
-          <t>3000 m hinder</t>
+          <t>5000 m</t>
         </is>
       </c>
       <c r="H188" s="7" t="inlineStr">
         <is>
-          <t>9:40.58</t>
+          <t>15:23.39</t>
         </is>
       </c>
       <c r="I188" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J188" s="7" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PB, norsk U23-rekord</t>
         </is>
       </c>
     </row>
@@ -30248,7 +30248,7 @@
       </c>
       <c r="D592" s="7" t="inlineStr">
         <is>
-          <t>Riley McGown</t>
+          <t>Ulrik Moen Ødegård</t>
         </is>
       </c>
       <c r="E592" s="6" t="inlineStr">
@@ -30263,12 +30263,12 @@
       </c>
       <c r="G592" s="6" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>10000 m</t>
         </is>
       </c>
       <c r="H592" s="7" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>32:20.55</t>
         </is>
       </c>
       <c r="I592" s="7" t="inlineStr">
@@ -30278,7 +30278,7 @@
       </c>
       <c r="J592" s="7" t="inlineStr">
         <is>
-          <t>heat 2</t>
+          <t>elite</t>
         </is>
       </c>
     </row>
@@ -30300,37 +30300,37 @@
       </c>
       <c r="D593" s="7" t="inlineStr">
         <is>
-          <t>Henning Hellebust</t>
+          <t>Catherine Synnøve Vaugelade Berg</t>
         </is>
       </c>
       <c r="E593" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F593" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G593" s="6" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>10000 m</t>
         </is>
       </c>
       <c r="H593" s="7" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>37:06.44</t>
         </is>
       </c>
       <c r="I593" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J593" s="7" t="inlineStr">
         <is>
-          <t>heat 2</t>
+          <t>elite</t>
         </is>
       </c>
     </row>
@@ -30352,37 +30352,37 @@
       </c>
       <c r="D594" s="7" t="inlineStr">
         <is>
-          <t>Aleksander Amundsen</t>
+          <t>Andrea Langmo</t>
         </is>
       </c>
       <c r="E594" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F594" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G594" s="6" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>10000 m</t>
         </is>
       </c>
       <c r="H594" s="7" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>38:24.90</t>
         </is>
       </c>
       <c r="I594" s="7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J594" s="7" t="inlineStr">
         <is>
-          <t>heat 2</t>
+          <t>elite</t>
         </is>
       </c>
     </row>
@@ -30404,7 +30404,7 @@
       </c>
       <c r="D595" s="7" t="inlineStr">
         <is>
-          <t>Gjermund Fluge Ulleberg</t>
+          <t>Riley McGown</t>
         </is>
       </c>
       <c r="E595" s="6" t="inlineStr">
@@ -30424,12 +30424,12 @@
       </c>
       <c r="H595" s="7" t="inlineStr">
         <is>
-          <t>17:17</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="I595" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J595" s="7" t="inlineStr">
@@ -30456,17 +30456,17 @@
       </c>
       <c r="D596" s="7" t="inlineStr">
         <is>
-          <t>Selma Størmer-Antonsen</t>
+          <t>Henning Hellebust</t>
         </is>
       </c>
       <c r="E596" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F596" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G596" s="6" t="inlineStr">
@@ -30476,12 +30476,12 @@
       </c>
       <c r="H596" s="7" t="inlineStr">
         <is>
-          <t>17:33</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="I596" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J596" s="7" t="inlineStr">
@@ -30508,7 +30508,7 @@
       </c>
       <c r="D597" s="7" t="inlineStr">
         <is>
-          <t>Lars Gellein Halvorsen</t>
+          <t>Aleksander Amundsen</t>
         </is>
       </c>
       <c r="E597" s="6" t="inlineStr">
@@ -30528,12 +30528,12 @@
       </c>
       <c r="H597" s="7" t="inlineStr">
         <is>
-          <t>18:14</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I597" s="7" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J597" s="7" t="inlineStr">
@@ -30560,7 +30560,7 @@
       </c>
       <c r="D598" s="7" t="inlineStr">
         <is>
-          <t>Jan Petter Mork</t>
+          <t>Gjermund Fluge Ulleberg</t>
         </is>
       </c>
       <c r="E598" s="6" t="inlineStr">
@@ -30580,12 +30580,12 @@
       </c>
       <c r="H598" s="7" t="inlineStr">
         <is>
-          <t>18:17</t>
+          <t>17:17</t>
         </is>
       </c>
       <c r="I598" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J598" s="7" t="inlineStr">
@@ -30612,7 +30612,7 @@
       </c>
       <c r="D599" s="7" t="inlineStr">
         <is>
-          <t>Jessica Gunnarsson</t>
+          <t>Selma Størmer-Antonsen</t>
         </is>
       </c>
       <c r="E599" s="6" t="inlineStr">
@@ -30632,17 +30632,17 @@
       </c>
       <c r="H599" s="7" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="I599" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J599" s="7" t="inlineStr">
         <is>
-          <t>heat 1</t>
+          <t>heat 2</t>
         </is>
       </c>
     </row>
@@ -30664,7 +30664,7 @@
       </c>
       <c r="D600" s="7" t="inlineStr">
         <is>
-          <t>Jo Trieu</t>
+          <t>Lars Gellein Halvorsen</t>
         </is>
       </c>
       <c r="E600" s="6" t="inlineStr">
@@ -30684,17 +30684,17 @@
       </c>
       <c r="H600" s="7" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>18:14</t>
         </is>
       </c>
       <c r="I600" s="7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J600" s="7" t="inlineStr">
         <is>
-          <t>heat 1</t>
+          <t>heat 2</t>
         </is>
       </c>
     </row>
@@ -30716,17 +30716,17 @@
       </c>
       <c r="D601" s="7" t="inlineStr">
         <is>
-          <t>Mathilde Nordahl</t>
+          <t>Jan Petter Mork</t>
         </is>
       </c>
       <c r="E601" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F601" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G601" s="6" t="inlineStr">
@@ -30736,17 +30736,17 @@
       </c>
       <c r="H601" s="7" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>18:17</t>
         </is>
       </c>
       <c r="I601" s="7" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>21</t>
         </is>
       </c>
       <c r="J601" s="7" t="inlineStr">
         <is>
-          <t>heat 1</t>
+          <t>heat 2</t>
         </is>
       </c>
     </row>
@@ -30768,7 +30768,7 @@
       </c>
       <c r="D602" s="7" t="inlineStr">
         <is>
-          <t>Jenny Lillehagen Garnes</t>
+          <t>Jessica Gunnarsson</t>
         </is>
       </c>
       <c r="E602" s="6" t="inlineStr">
@@ -30788,12 +30788,12 @@
       </c>
       <c r="H602" s="7" t="inlineStr">
         <is>
-          <t>22:23</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="I602" s="7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J602" s="7" t="inlineStr">
@@ -30820,7 +30820,7 @@
       </c>
       <c r="D603" s="7" t="inlineStr">
         <is>
-          <t>Martin Kjäll-Ohlsson</t>
+          <t>Jo Trieu</t>
         </is>
       </c>
       <c r="E603" s="6" t="inlineStr">
@@ -30835,22 +30835,22 @@
       </c>
       <c r="G603" s="6" t="inlineStr">
         <is>
-          <t>10 km</t>
+          <t>5 km</t>
         </is>
       </c>
       <c r="H603" s="7" t="inlineStr">
         <is>
-          <t>33:27</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="I603" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J603" s="7" t="inlineStr">
         <is>
-          <t>heat 2</t>
+          <t>heat 1</t>
         </is>
       </c>
     </row>
@@ -30872,37 +30872,37 @@
       </c>
       <c r="D604" s="7" t="inlineStr">
         <is>
-          <t>Tobias Gram-Caspersen</t>
+          <t>Mathilde Nordahl</t>
         </is>
       </c>
       <c r="E604" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F604" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G604" s="6" t="inlineStr">
         <is>
-          <t>10 km</t>
+          <t>5 km</t>
         </is>
       </c>
       <c r="H604" s="7" t="inlineStr">
         <is>
-          <t>34:08</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="I604" s="7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>14</t>
         </is>
       </c>
       <c r="J604" s="7" t="inlineStr">
         <is>
-          <t>heat 2</t>
+          <t>heat 1</t>
         </is>
       </c>
     </row>
@@ -30924,37 +30924,37 @@
       </c>
       <c r="D605" s="7" t="inlineStr">
         <is>
-          <t>Eivind Bækkedal</t>
+          <t>Jenny Lillehagen Garnes</t>
         </is>
       </c>
       <c r="E605" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F605" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G605" s="6" t="inlineStr">
         <is>
-          <t>10 km</t>
+          <t>5 km</t>
         </is>
       </c>
       <c r="H605" s="7" t="inlineStr">
         <is>
-          <t>35:04</t>
+          <t>22:23</t>
         </is>
       </c>
       <c r="I605" s="7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="J605" s="7" t="inlineStr">
         <is>
-          <t>heat 2</t>
+          <t>heat 1</t>
         </is>
       </c>
     </row>
@@ -30976,7 +30976,7 @@
       </c>
       <c r="D606" s="7" t="inlineStr">
         <is>
-          <t>Jacob Nitter</t>
+          <t>Martin Kjäll-Ohlsson</t>
         </is>
       </c>
       <c r="E606" s="6" t="inlineStr">
@@ -30996,12 +30996,12 @@
       </c>
       <c r="H606" s="7" t="inlineStr">
         <is>
-          <t>35:38</t>
+          <t>33:27</t>
         </is>
       </c>
       <c r="I606" s="7" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J606" s="7" t="inlineStr">
@@ -31028,7 +31028,7 @@
       </c>
       <c r="D607" s="7" t="inlineStr">
         <is>
-          <t>Aksel Petter Spence</t>
+          <t>Tobias Gram-Caspersen</t>
         </is>
       </c>
       <c r="E607" s="6" t="inlineStr">
@@ -31048,12 +31048,12 @@
       </c>
       <c r="H607" s="7" t="inlineStr">
         <is>
-          <t>35:57</t>
+          <t>34:08</t>
         </is>
       </c>
       <c r="I607" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4</t>
         </is>
       </c>
       <c r="J607" s="7" t="inlineStr">
@@ -31080,7 +31080,7 @@
       </c>
       <c r="D608" s="7" t="inlineStr">
         <is>
-          <t>Andreas Solheim</t>
+          <t>Eivind Bækkedal</t>
         </is>
       </c>
       <c r="E608" s="6" t="inlineStr">
@@ -31100,12 +31100,12 @@
       </c>
       <c r="H608" s="7" t="inlineStr">
         <is>
-          <t>35:59</t>
+          <t>35:04</t>
         </is>
       </c>
       <c r="I608" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="J608" s="7" t="inlineStr">
@@ -31132,7 +31132,7 @@
       </c>
       <c r="D609" s="7" t="inlineStr">
         <is>
-          <t>Bjørnar Kjønnøy Slettvåg</t>
+          <t>Jacob Nitter</t>
         </is>
       </c>
       <c r="E609" s="6" t="inlineStr">
@@ -31152,12 +31152,12 @@
       </c>
       <c r="H609" s="7" t="inlineStr">
         <is>
-          <t>37:24</t>
+          <t>35:38</t>
         </is>
       </c>
       <c r="I609" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>6</t>
         </is>
       </c>
       <c r="J609" s="7" t="inlineStr">
@@ -31184,7 +31184,7 @@
       </c>
       <c r="D610" s="7" t="inlineStr">
         <is>
-          <t>Sven Thelin</t>
+          <t>Aksel Petter Spence</t>
         </is>
       </c>
       <c r="E610" s="6" t="inlineStr">
@@ -31204,12 +31204,12 @@
       </c>
       <c r="H610" s="7" t="inlineStr">
         <is>
-          <t>37:24</t>
+          <t>35:57</t>
         </is>
       </c>
       <c r="I610" s="7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J610" s="7" t="inlineStr">
@@ -31236,17 +31236,17 @@
       </c>
       <c r="D611" s="7" t="inlineStr">
         <is>
-          <t>Torill Ytterhus Haugset</t>
+          <t>Andreas Solheim</t>
         </is>
       </c>
       <c r="E611" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F611" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G611" s="6" t="inlineStr">
@@ -31256,17 +31256,17 @@
       </c>
       <c r="H611" s="7" t="inlineStr">
         <is>
-          <t>41:06</t>
+          <t>35:59</t>
         </is>
       </c>
       <c r="I611" s="7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J611" s="7" t="inlineStr">
         <is>
-          <t>heat 1</t>
+          <t>heat 2</t>
         </is>
       </c>
     </row>
@@ -31288,17 +31288,17 @@
       </c>
       <c r="D612" s="7" t="inlineStr">
         <is>
-          <t>Marte Solset Haug</t>
+          <t>Bjørnar Kjønnøy Slettvåg</t>
         </is>
       </c>
       <c r="E612" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F612" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G612" s="6" t="inlineStr">
@@ -31308,17 +31308,17 @@
       </c>
       <c r="H612" s="7" t="inlineStr">
         <is>
-          <t>41:34</t>
+          <t>37:24</t>
         </is>
       </c>
       <c r="I612" s="7" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J612" s="7" t="inlineStr">
         <is>
-          <t>heat 1</t>
+          <t>heat 2</t>
         </is>
       </c>
     </row>
@@ -31340,17 +31340,17 @@
       </c>
       <c r="D613" s="7" t="inlineStr">
         <is>
-          <t>Live Maria Grønvold</t>
+          <t>Sven Thelin</t>
         </is>
       </c>
       <c r="E613" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F613" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G613" s="6" t="inlineStr">
@@ -31360,17 +31360,17 @@
       </c>
       <c r="H613" s="7" t="inlineStr">
         <is>
-          <t>42:02</t>
+          <t>37:24</t>
         </is>
       </c>
       <c r="I613" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J613" s="7" t="inlineStr">
         <is>
-          <t>heat 1</t>
+          <t>heat 2</t>
         </is>
       </c>
     </row>
@@ -31392,17 +31392,17 @@
       </c>
       <c r="D614" s="7" t="inlineStr">
         <is>
-          <t>Daniel Espedokken Severinsen</t>
+          <t>Torill Ytterhus Haugset</t>
         </is>
       </c>
       <c r="E614" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F614" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G614" s="6" t="inlineStr">
@@ -31412,12 +31412,12 @@
       </c>
       <c r="H614" s="7" t="inlineStr">
         <is>
-          <t>42:03</t>
+          <t>41:06</t>
         </is>
       </c>
       <c r="I614" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>7</t>
         </is>
       </c>
       <c r="J614" s="7" t="inlineStr">
@@ -31444,17 +31444,17 @@
       </c>
       <c r="D615" s="7" t="inlineStr">
         <is>
-          <t>Bjarni Herrera Thorisson</t>
+          <t>Marte Solset Haug</t>
         </is>
       </c>
       <c r="E615" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F615" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G615" s="6" t="inlineStr">
@@ -31464,12 +31464,12 @@
       </c>
       <c r="H615" s="7" t="inlineStr">
         <is>
-          <t>45:45</t>
+          <t>41:34</t>
         </is>
       </c>
       <c r="I615" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="J615" s="7" t="inlineStr">
@@ -31496,17 +31496,17 @@
       </c>
       <c r="D616" s="7" t="inlineStr">
         <is>
-          <t>Eirik Haugland Kvalvik</t>
+          <t>Live Maria Grønvold</t>
         </is>
       </c>
       <c r="E616" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F616" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G616" s="6" t="inlineStr">
@@ -31516,12 +31516,12 @@
       </c>
       <c r="H616" s="7" t="inlineStr">
         <is>
-          <t>46:38</t>
+          <t>42:02</t>
         </is>
       </c>
       <c r="I616" s="7" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>10</t>
         </is>
       </c>
       <c r="J616" s="7" t="inlineStr">
@@ -31548,7 +31548,7 @@
       </c>
       <c r="D617" s="7" t="inlineStr">
         <is>
-          <t>Ulrik Moen Ødegård</t>
+          <t>Daniel Espedokken Severinsen</t>
         </is>
       </c>
       <c r="E617" s="6" t="inlineStr">
@@ -31563,22 +31563,22 @@
       </c>
       <c r="G617" s="6" t="inlineStr">
         <is>
-          <t>10000 m</t>
+          <t>10 km</t>
         </is>
       </c>
       <c r="H617" s="7" t="inlineStr">
         <is>
-          <t>32:20.55</t>
+          <t>42:03</t>
         </is>
       </c>
       <c r="I617" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J617" s="7" t="inlineStr">
         <is>
-          <t>elite</t>
+          <t>heat 1</t>
         </is>
       </c>
     </row>
@@ -31600,37 +31600,37 @@
       </c>
       <c r="D618" s="7" t="inlineStr">
         <is>
-          <t>Catherine Synnøve Vaugelade Berg</t>
+          <t>Bjarni Herrera Thorisson</t>
         </is>
       </c>
       <c r="E618" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F618" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G618" s="6" t="inlineStr">
         <is>
-          <t>10000 m</t>
+          <t>10 km</t>
         </is>
       </c>
       <c r="H618" s="7" t="inlineStr">
         <is>
-          <t>37:06.44</t>
+          <t>45:45</t>
         </is>
       </c>
       <c r="I618" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J618" s="7" t="inlineStr">
         <is>
-          <t>elite</t>
+          <t>heat 1</t>
         </is>
       </c>
     </row>
@@ -31652,37 +31652,37 @@
       </c>
       <c r="D619" s="7" t="inlineStr">
         <is>
-          <t>Andrea Langmo</t>
+          <t>Eirik Haugland Kvalvik</t>
         </is>
       </c>
       <c r="E619" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F619" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G619" s="6" t="inlineStr">
         <is>
-          <t>10000 m</t>
+          <t>10 km</t>
         </is>
       </c>
       <c r="H619" s="7" t="inlineStr">
         <is>
-          <t>38:24.90</t>
+          <t>46:38</t>
         </is>
       </c>
       <c r="I619" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>19</t>
         </is>
       </c>
       <c r="J619" s="7" t="inlineStr">
         <is>
-          <t>elite</t>
+          <t>heat 1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Kristiansund Havmaraton distance
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -3127,7 +3127,7 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>Maraton</t>
+          <t>Halvmaraton</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1</t>
+          <t>1. kvinne, klasse 1; rettet fra Havmaraton til Halvmaraton</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Espen Bielke New Delhi half marathon result
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -202,8 +202,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VidarLangdistanse" displayName="VidarLangdistanse" ref="A8:J1409" headerRowCount="1">
-  <autoFilter ref="A8:J1409"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VidarLangdistanse" displayName="VidarLangdistanse" ref="A8:J1410" headerRowCount="1">
+  <autoFilter ref="A8:J1410"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Uke"/>
     <tableColumn id="2" name="Dato"/>
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1409"/>
+  <dimension ref="A1:J1410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -576,13 +576,13 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>1401</v>
+        <v>1402</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>567</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -64349,22 +64349,22 @@
     <row r="1293">
       <c r="A1293" s="6" t="inlineStr">
         <is>
-          <t>Uke 7</t>
+          <t>Uke 8</t>
         </is>
       </c>
       <c r="B1293" s="6" t="inlineStr">
         <is>
-          <t>15.02.2026</t>
+          <t>22.02.2026</t>
         </is>
       </c>
       <c r="C1293" s="7" t="inlineStr">
         <is>
-          <t>Barcelona Halvmaraton</t>
+          <t>New Delhi Half Marathon 2026</t>
         </is>
       </c>
       <c r="D1293" s="7" t="inlineStr">
         <is>
-          <t>Sjur Prestsæter</t>
+          <t>Espen Bielke</t>
         </is>
       </c>
       <c r="E1293" s="6" t="inlineStr">
@@ -64374,7 +64374,7 @@
       </c>
       <c r="F1293" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>Menn</t>
         </is>
       </c>
       <c r="G1293" s="6" t="inlineStr">
@@ -64384,17 +64384,13 @@
       </c>
       <c r="H1293" s="7" t="inlineStr">
         <is>
-          <t>01:03:13</t>
-        </is>
-      </c>
-      <c r="I1293" s="7" t="inlineStr">
-        <is>
-          <t>39</t>
-        </is>
-      </c>
+          <t>1:36:08</t>
+        </is>
+      </c>
+      <c r="I1293" s="7" t="inlineStr"/>
       <c r="J1293" s="7" t="inlineStr">
         <is>
-          <t>M pos: 39</t>
+          <t>Foreløpig resultat, startnummer 2001, Defence Colony Tehsil, India, RaceTime India SMS</t>
         </is>
       </c>
     </row>
@@ -64416,7 +64412,7 @@
       </c>
       <c r="D1294" s="7" t="inlineStr">
         <is>
-          <t>Trond Einar Moen Pedersli</t>
+          <t>Sjur Prestsæter</t>
         </is>
       </c>
       <c r="E1294" s="6" t="inlineStr">
@@ -64436,17 +64432,17 @@
       </c>
       <c r="H1294" s="7" t="inlineStr">
         <is>
-          <t>01:05:46</t>
+          <t>01:03:13</t>
         </is>
       </c>
       <c r="I1294" s="7" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>39</t>
         </is>
       </c>
       <c r="J1294" s="7" t="inlineStr">
         <is>
-          <t>M pos: 90</t>
+          <t>M pos: 39</t>
         </is>
       </c>
     </row>
@@ -64468,7 +64464,7 @@
       </c>
       <c r="D1295" s="7" t="inlineStr">
         <is>
-          <t>Sondre Lomeland</t>
+          <t>Trond Einar Moen Pedersli</t>
         </is>
       </c>
       <c r="E1295" s="6" t="inlineStr">
@@ -64488,17 +64484,17 @@
       </c>
       <c r="H1295" s="7" t="inlineStr">
         <is>
-          <t>01:06:44</t>
+          <t>01:05:46</t>
         </is>
       </c>
       <c r="I1295" s="7" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>90</t>
         </is>
       </c>
       <c r="J1295" s="7" t="inlineStr">
         <is>
-          <t>M pos: 116</t>
+          <t>M pos: 90</t>
         </is>
       </c>
     </row>
@@ -64520,7 +64516,7 @@
       </c>
       <c r="D1296" s="7" t="inlineStr">
         <is>
-          <t>Martin Finne</t>
+          <t>Sondre Lomeland</t>
         </is>
       </c>
       <c r="E1296" s="6" t="inlineStr">
@@ -64540,17 +64536,17 @@
       </c>
       <c r="H1296" s="7" t="inlineStr">
         <is>
-          <t>01:08:51</t>
+          <t>01:06:44</t>
         </is>
       </c>
       <c r="I1296" s="7" t="inlineStr">
         <is>
-          <t>176</t>
+          <t>116</t>
         </is>
       </c>
       <c r="J1296" s="7" t="inlineStr">
         <is>
-          <t>M pos: 176</t>
+          <t>M pos: 116</t>
         </is>
       </c>
     </row>
@@ -64572,7 +64568,7 @@
       </c>
       <c r="D1297" s="7" t="inlineStr">
         <is>
-          <t>Morten Dalhaug</t>
+          <t>Martin Finne</t>
         </is>
       </c>
       <c r="E1297" s="6" t="inlineStr">
@@ -64592,17 +64588,17 @@
       </c>
       <c r="H1297" s="7" t="inlineStr">
         <is>
-          <t>01:10:14</t>
+          <t>01:08:51</t>
         </is>
       </c>
       <c r="I1297" s="7" t="inlineStr">
         <is>
-          <t>250</t>
+          <t>176</t>
         </is>
       </c>
       <c r="J1297" s="7" t="inlineStr">
         <is>
-          <t>M pos: 250</t>
+          <t>M pos: 176</t>
         </is>
       </c>
     </row>
@@ -64624,17 +64620,17 @@
       </c>
       <c r="D1298" s="7" t="inlineStr">
         <is>
-          <t>Ingrid Helene Nyhus</t>
+          <t>Morten Dalhaug</t>
         </is>
       </c>
       <c r="E1298" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1298" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1298" s="6" t="inlineStr">
@@ -64644,17 +64640,17 @@
       </c>
       <c r="H1298" s="7" t="inlineStr">
         <is>
-          <t>01:16:27</t>
+          <t>01:10:14</t>
         </is>
       </c>
       <c r="I1298" s="7" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>250</t>
         </is>
       </c>
       <c r="J1298" s="7" t="inlineStr">
         <is>
-          <t>K pos: 51</t>
+          <t>M pos: 250</t>
         </is>
       </c>
     </row>
@@ -64676,17 +64672,17 @@
       </c>
       <c r="D1299" s="7" t="inlineStr">
         <is>
-          <t>Henrik Victor Hansen</t>
+          <t>Ingrid Helene Nyhus</t>
         </is>
       </c>
       <c r="E1299" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1299" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1299" s="6" t="inlineStr">
@@ -64696,11 +64692,19 @@
       </c>
       <c r="H1299" s="7" t="inlineStr">
         <is>
-          <t>01:16:47</t>
-        </is>
-      </c>
-      <c r="I1299" s="7" t="inlineStr"/>
-      <c r="J1299" s="7" t="inlineStr"/>
+          <t>01:16:27</t>
+        </is>
+      </c>
+      <c r="I1299" s="7" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="J1299" s="7" t="inlineStr">
+        <is>
+          <t>K pos: 51</t>
+        </is>
+      </c>
     </row>
     <row r="1300">
       <c r="A1300" s="6" t="inlineStr">
@@ -64720,7 +64724,7 @@
       </c>
       <c r="D1300" s="7" t="inlineStr">
         <is>
-          <t>Jakov Semaskevic</t>
+          <t>Henrik Victor Hansen</t>
         </is>
       </c>
       <c r="E1300" s="6" t="inlineStr">
@@ -64740,7 +64744,7 @@
       </c>
       <c r="H1300" s="7" t="inlineStr">
         <is>
-          <t>01:18:42</t>
+          <t>01:16:47</t>
         </is>
       </c>
       <c r="I1300" s="7" t="inlineStr"/>
@@ -64764,7 +64768,7 @@
       </c>
       <c r="D1301" s="7" t="inlineStr">
         <is>
-          <t>Even Lund</t>
+          <t>Jakov Semaskevic</t>
         </is>
       </c>
       <c r="E1301" s="6" t="inlineStr">
@@ -64784,7 +64788,7 @@
       </c>
       <c r="H1301" s="7" t="inlineStr">
         <is>
-          <t>01:21:26</t>
+          <t>01:18:42</t>
         </is>
       </c>
       <c r="I1301" s="7" t="inlineStr"/>
@@ -64808,7 +64812,7 @@
       </c>
       <c r="D1302" s="7" t="inlineStr">
         <is>
-          <t>Erlend Bruaset</t>
+          <t>Even Lund</t>
         </is>
       </c>
       <c r="E1302" s="6" t="inlineStr">
@@ -64828,7 +64832,7 @@
       </c>
       <c r="H1302" s="7" t="inlineStr">
         <is>
-          <t>01:21:39</t>
+          <t>01:21:26</t>
         </is>
       </c>
       <c r="I1302" s="7" t="inlineStr"/>
@@ -64852,7 +64856,7 @@
       </c>
       <c r="D1303" s="7" t="inlineStr">
         <is>
-          <t>Benjamin Hai Duong</t>
+          <t>Erlend Bruaset</t>
         </is>
       </c>
       <c r="E1303" s="6" t="inlineStr">
@@ -64872,7 +64876,7 @@
       </c>
       <c r="H1303" s="7" t="inlineStr">
         <is>
-          <t>01:21:53</t>
+          <t>01:21:39</t>
         </is>
       </c>
       <c r="I1303" s="7" t="inlineStr"/>
@@ -64896,7 +64900,7 @@
       </c>
       <c r="D1304" s="7" t="inlineStr">
         <is>
-          <t>John Fuller</t>
+          <t>Benjamin Hai Duong</t>
         </is>
       </c>
       <c r="E1304" s="6" t="inlineStr">
@@ -64916,7 +64920,7 @@
       </c>
       <c r="H1304" s="7" t="inlineStr">
         <is>
-          <t>01:25:30</t>
+          <t>01:21:53</t>
         </is>
       </c>
       <c r="I1304" s="7" t="inlineStr"/>
@@ -64940,7 +64944,7 @@
       </c>
       <c r="D1305" s="7" t="inlineStr">
         <is>
-          <t>Andreas Sung Unstad</t>
+          <t>John Fuller</t>
         </is>
       </c>
       <c r="E1305" s="6" t="inlineStr">
@@ -64960,7 +64964,7 @@
       </c>
       <c r="H1305" s="7" t="inlineStr">
         <is>
-          <t>01:29:16</t>
+          <t>01:25:30</t>
         </is>
       </c>
       <c r="I1305" s="7" t="inlineStr"/>
@@ -64984,17 +64988,17 @@
       </c>
       <c r="D1306" s="7" t="inlineStr">
         <is>
-          <t>Mari Vatn</t>
+          <t>Andreas Sung Unstad</t>
         </is>
       </c>
       <c r="E1306" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1306" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1306" s="6" t="inlineStr">
@@ -65004,7 +65008,7 @@
       </c>
       <c r="H1306" s="7" t="inlineStr">
         <is>
-          <t>01:38:49</t>
+          <t>01:29:16</t>
         </is>
       </c>
       <c r="I1306" s="7" t="inlineStr"/>
@@ -65028,7 +65032,7 @@
       </c>
       <c r="D1307" s="7" t="inlineStr">
         <is>
-          <t>Julie Didriksen</t>
+          <t>Mari Vatn</t>
         </is>
       </c>
       <c r="E1307" s="6" t="inlineStr">
@@ -65048,7 +65052,7 @@
       </c>
       <c r="H1307" s="7" t="inlineStr">
         <is>
-          <t>01:44:08</t>
+          <t>01:38:49</t>
         </is>
       </c>
       <c r="I1307" s="7" t="inlineStr"/>
@@ -65067,12 +65071,12 @@
       </c>
       <c r="C1308" s="7" t="inlineStr">
         <is>
-          <t>Monaco 5k</t>
+          <t>Barcelona Halvmaraton</t>
         </is>
       </c>
       <c r="D1308" s="7" t="inlineStr">
         <is>
-          <t>Amalie Sæten</t>
+          <t>Julie Didriksen</t>
         </is>
       </c>
       <c r="E1308" s="6" t="inlineStr">
@@ -65087,12 +65091,12 @@
       </c>
       <c r="G1308" s="6" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>Halvmaraton</t>
         </is>
       </c>
       <c r="H1308" s="7" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>01:44:08</t>
         </is>
       </c>
       <c r="I1308" s="7" t="inlineStr"/>
@@ -65116,17 +65120,17 @@
       </c>
       <c r="D1309" s="7" t="inlineStr">
         <is>
-          <t>Ådne Andersen</t>
+          <t>Amalie Sæten</t>
         </is>
       </c>
       <c r="E1309" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1309" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1309" s="6" t="inlineStr">
@@ -65136,15 +65140,11 @@
       </c>
       <c r="H1309" s="7" t="inlineStr">
         <is>
-          <t>15:29</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="I1309" s="7" t="inlineStr"/>
-      <c r="J1309" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1309" s="7" t="inlineStr"/>
     </row>
     <row r="1310">
       <c r="A1310" s="6" t="inlineStr">
@@ -65164,17 +65164,17 @@
       </c>
       <c r="D1310" s="7" t="inlineStr">
         <is>
-          <t>Ine Bakken</t>
+          <t>Ådne Andersen</t>
         </is>
       </c>
       <c r="E1310" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1310" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1310" s="6" t="inlineStr">
@@ -65184,11 +65184,15 @@
       </c>
       <c r="H1310" s="7" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>15:29</t>
         </is>
       </c>
       <c r="I1310" s="7" t="inlineStr"/>
-      <c r="J1310" s="7" t="inlineStr"/>
+      <c r="J1310" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1311">
       <c r="A1311" s="6" t="inlineStr">
@@ -65203,32 +65207,32 @@
       </c>
       <c r="C1311" s="7" t="inlineStr">
         <is>
-          <t>Sevilla Maraton</t>
+          <t>Monaco 5k</t>
         </is>
       </c>
       <c r="D1311" s="7" t="inlineStr">
         <is>
-          <t>Aleksander</t>
+          <t>Ine Bakken</t>
         </is>
       </c>
       <c r="E1311" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1311" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1311" s="6" t="inlineStr">
         <is>
-          <t>Maraton</t>
+          <t>5 km</t>
         </is>
       </c>
       <c r="H1311" s="7" t="inlineStr">
         <is>
-          <t>2:42:30</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="I1311" s="7" t="inlineStr"/>
@@ -65252,7 +65256,7 @@
       </c>
       <c r="D1312" s="7" t="inlineStr">
         <is>
-          <t>Marius Borkenhagen</t>
+          <t>Aleksander</t>
         </is>
       </c>
       <c r="E1312" s="6" t="inlineStr">
@@ -65272,7 +65276,7 @@
       </c>
       <c r="H1312" s="7" t="inlineStr">
         <is>
-          <t>02:54:04</t>
+          <t>2:42:30</t>
         </is>
       </c>
       <c r="I1312" s="7" t="inlineStr"/>
@@ -65296,7 +65300,7 @@
       </c>
       <c r="D1313" s="7" t="inlineStr">
         <is>
-          <t>Anders Nordby</t>
+          <t>Marius Borkenhagen</t>
         </is>
       </c>
       <c r="E1313" s="6" t="inlineStr">
@@ -65316,7 +65320,7 @@
       </c>
       <c r="H1313" s="7" t="inlineStr">
         <is>
-          <t>03:06:48</t>
+          <t>02:54:04</t>
         </is>
       </c>
       <c r="I1313" s="7" t="inlineStr"/>
@@ -65340,7 +65344,7 @@
       </c>
       <c r="D1314" s="7" t="inlineStr">
         <is>
-          <t>Ole Jørgen Jacobsen</t>
+          <t>Anders Nordby</t>
         </is>
       </c>
       <c r="E1314" s="6" t="inlineStr">
@@ -65360,7 +65364,7 @@
       </c>
       <c r="H1314" s="7" t="inlineStr">
         <is>
-          <t>03:21:32</t>
+          <t>03:06:48</t>
         </is>
       </c>
       <c r="I1314" s="7" t="inlineStr"/>
@@ -65384,7 +65388,7 @@
       </c>
       <c r="D1315" s="7" t="inlineStr">
         <is>
-          <t>Fredrik Camilo Halsbog</t>
+          <t>Ole Jørgen Jacobsen</t>
         </is>
       </c>
       <c r="E1315" s="6" t="inlineStr">
@@ -65404,7 +65408,7 @@
       </c>
       <c r="H1315" s="7" t="inlineStr">
         <is>
-          <t>03:35:22</t>
+          <t>03:21:32</t>
         </is>
       </c>
       <c r="I1315" s="7" t="inlineStr"/>
@@ -65423,90 +65427,82 @@
       </c>
       <c r="C1316" s="7" t="inlineStr">
         <is>
-          <t>Sierra Blanca Trail - Destroyer 42k</t>
+          <t>Sevilla Maraton</t>
         </is>
       </c>
       <c r="D1316" s="7" t="inlineStr">
         <is>
-          <t>Maria Bipop</t>
+          <t>Fredrik Camilo Halsbog</t>
         </is>
       </c>
       <c r="E1316" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1316" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1316" s="6" t="inlineStr">
         <is>
-          <t>42 km</t>
-        </is>
-      </c>
-      <c r="H1316" s="7" t="inlineStr"/>
-      <c r="I1316" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="J1316" s="7" t="inlineStr">
-        <is>
-          <t>2. plass</t>
-        </is>
-      </c>
+          <t>Maraton</t>
+        </is>
+      </c>
+      <c r="H1316" s="7" t="inlineStr">
+        <is>
+          <t>03:35:22</t>
+        </is>
+      </c>
+      <c r="I1316" s="7" t="inlineStr"/>
+      <c r="J1316" s="7" t="inlineStr"/>
     </row>
     <row r="1317">
       <c r="A1317" s="6" t="inlineStr">
         <is>
-          <t>Uke 6</t>
+          <t>Uke 7</t>
         </is>
       </c>
       <c r="B1317" s="6" t="inlineStr">
         <is>
-          <t>08.02.2026</t>
+          <t>15.02.2026</t>
         </is>
       </c>
       <c r="C1317" s="7" t="inlineStr">
         <is>
-          <t>Bislett Indoor Marathon</t>
+          <t>Sierra Blanca Trail - Destroyer 42k</t>
         </is>
       </c>
       <c r="D1317" s="7" t="inlineStr">
         <is>
-          <t>David Meier</t>
+          <t>Maria Bipop</t>
         </is>
       </c>
       <c r="E1317" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1317" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1317" s="6" t="inlineStr">
         <is>
-          <t>5 km</t>
-        </is>
-      </c>
-      <c r="H1317" s="7" t="inlineStr">
-        <is>
-          <t>14:51</t>
-        </is>
-      </c>
+          <t>42 km</t>
+        </is>
+      </c>
+      <c r="H1317" s="7" t="inlineStr"/>
       <c r="I1317" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J1317" s="7" t="inlineStr">
         <is>
-          <t>1. plass</t>
+          <t>2. plass</t>
         </is>
       </c>
     </row>
@@ -65528,7 +65524,7 @@
       </c>
       <c r="D1318" s="7" t="inlineStr">
         <is>
-          <t>Ådne Andersen</t>
+          <t>David Meier</t>
         </is>
       </c>
       <c r="E1318" s="6" t="inlineStr">
@@ -65548,13 +65544,17 @@
       </c>
       <c r="H1318" s="7" t="inlineStr">
         <is>
-          <t>15:12</t>
-        </is>
-      </c>
-      <c r="I1318" s="7" t="inlineStr"/>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="I1318" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="J1318" s="7" t="inlineStr">
         <is>
-          <t>fartsholder</t>
+          <t>1. plass</t>
         </is>
       </c>
     </row>
@@ -65576,7 +65576,7 @@
       </c>
       <c r="D1319" s="7" t="inlineStr">
         <is>
-          <t>Gaute Olberg</t>
+          <t>Ådne Andersen</t>
         </is>
       </c>
       <c r="E1319" s="6" t="inlineStr">
@@ -65596,11 +65596,15 @@
       </c>
       <c r="H1319" s="7" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="I1319" s="7" t="inlineStr"/>
-      <c r="J1319" s="7" t="inlineStr"/>
+      <c r="J1319" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1320">
       <c r="A1320" s="6" t="inlineStr">
@@ -65620,7 +65624,7 @@
       </c>
       <c r="D1320" s="7" t="inlineStr">
         <is>
-          <t>Ådne Andersen</t>
+          <t>Gaute Olberg</t>
         </is>
       </c>
       <c r="E1320" s="6" t="inlineStr">
@@ -65640,15 +65644,11 @@
       </c>
       <c r="H1320" s="7" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="I1320" s="7" t="inlineStr"/>
-      <c r="J1320" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1320" s="7" t="inlineStr"/>
     </row>
     <row r="1321">
       <c r="A1321" s="6" t="inlineStr">
@@ -65668,17 +65668,17 @@
       </c>
       <c r="D1321" s="7" t="inlineStr">
         <is>
-          <t>Anna Marie Sirevåg</t>
+          <t>Ådne Andersen</t>
         </is>
       </c>
       <c r="E1321" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1321" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1321" s="6" t="inlineStr">
@@ -65688,17 +65688,13 @@
       </c>
       <c r="H1321" s="7" t="inlineStr">
         <is>
-          <t>15:42</t>
-        </is>
-      </c>
-      <c r="I1321" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="I1321" s="7" t="inlineStr"/>
       <c r="J1321" s="7" t="inlineStr">
         <is>
-          <t>1. plass</t>
+          <t>fartsholder</t>
         </is>
       </c>
     </row>
@@ -65720,17 +65716,17 @@
       </c>
       <c r="D1322" s="7" t="inlineStr">
         <is>
-          <t>Martin Kjäll-Ohlsson</t>
+          <t>Anna Marie Sirevåg</t>
         </is>
       </c>
       <c r="E1322" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1322" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1322" s="6" t="inlineStr">
@@ -65740,11 +65736,19 @@
       </c>
       <c r="H1322" s="7" t="inlineStr">
         <is>
-          <t>16:06</t>
-        </is>
-      </c>
-      <c r="I1322" s="7" t="inlineStr"/>
-      <c r="J1322" s="7" t="inlineStr"/>
+          <t>15:42</t>
+        </is>
+      </c>
+      <c r="I1322" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J1322" s="7" t="inlineStr">
+        <is>
+          <t>1. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1323">
       <c r="A1323" s="6" t="inlineStr">
@@ -65764,17 +65768,17 @@
       </c>
       <c r="D1323" s="7" t="inlineStr">
         <is>
-          <t>Emilie Mo</t>
+          <t>Martin Kjäll-Ohlsson</t>
         </is>
       </c>
       <c r="E1323" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1323" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1323" s="6" t="inlineStr">
@@ -65784,7 +65788,7 @@
       </c>
       <c r="H1323" s="7" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="I1323" s="7" t="inlineStr"/>
@@ -65808,17 +65812,17 @@
       </c>
       <c r="D1324" s="7" t="inlineStr">
         <is>
-          <t>Erlend Hellum</t>
+          <t>Emilie Mo</t>
         </is>
       </c>
       <c r="E1324" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1324" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1324" s="6" t="inlineStr">
@@ -65828,7 +65832,7 @@
       </c>
       <c r="H1324" s="7" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="I1324" s="7" t="inlineStr"/>
@@ -65852,17 +65856,17 @@
       </c>
       <c r="D1325" s="7" t="inlineStr">
         <is>
-          <t>Iben Kvigne</t>
+          <t>Erlend Hellum</t>
         </is>
       </c>
       <c r="E1325" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1325" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1325" s="6" t="inlineStr">
@@ -65872,19 +65876,11 @@
       </c>
       <c r="H1325" s="7" t="inlineStr">
         <is>
-          <t>17:24</t>
-        </is>
-      </c>
-      <c r="I1325" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="J1325" s="7" t="inlineStr">
-        <is>
-          <t>2. plass</t>
-        </is>
-      </c>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="I1325" s="7" t="inlineStr"/>
+      <c r="J1325" s="7" t="inlineStr"/>
     </row>
     <row r="1326">
       <c r="A1326" s="6" t="inlineStr">
@@ -65904,17 +65900,17 @@
       </c>
       <c r="D1326" s="7" t="inlineStr">
         <is>
-          <t>Nicolai Borenstein</t>
+          <t>Iben Kvigne</t>
         </is>
       </c>
       <c r="E1326" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1326" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1326" s="6" t="inlineStr">
@@ -65924,11 +65920,19 @@
       </c>
       <c r="H1326" s="7" t="inlineStr">
         <is>
-          <t>18:48</t>
-        </is>
-      </c>
-      <c r="I1326" s="7" t="inlineStr"/>
-      <c r="J1326" s="7" t="inlineStr"/>
+          <t>17:24</t>
+        </is>
+      </c>
+      <c r="I1326" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J1326" s="7" t="inlineStr">
+        <is>
+          <t>2. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1327">
       <c r="A1327" s="6" t="inlineStr">
@@ -65948,39 +65952,31 @@
       </c>
       <c r="D1327" s="7" t="inlineStr">
         <is>
-          <t>Liv Melby</t>
+          <t>Nicolai Borenstein</t>
         </is>
       </c>
       <c r="E1327" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1327" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1327" s="6" t="inlineStr">
         <is>
-          <t>10 km</t>
+          <t>5 km</t>
         </is>
       </c>
       <c r="H1327" s="7" t="inlineStr">
         <is>
-          <t>37:52</t>
-        </is>
-      </c>
-      <c r="I1327" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J1327" s="7" t="inlineStr">
-        <is>
-          <t>1. plass</t>
-        </is>
-      </c>
+          <t>18:48</t>
+        </is>
+      </c>
+      <c r="I1327" s="7" t="inlineStr"/>
+      <c r="J1327" s="7" t="inlineStr"/>
     </row>
     <row r="1328">
       <c r="A1328" s="6" t="inlineStr">
@@ -66000,31 +65996,39 @@
       </c>
       <c r="D1328" s="7" t="inlineStr">
         <is>
-          <t>Kristian Frøyen</t>
+          <t>Liv Melby</t>
         </is>
       </c>
       <c r="E1328" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1328" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1328" s="6" t="inlineStr">
         <is>
-          <t>Halvmaraton</t>
+          <t>10 km</t>
         </is>
       </c>
       <c r="H1328" s="7" t="inlineStr">
         <is>
-          <t>1:08:51</t>
-        </is>
-      </c>
-      <c r="I1328" s="7" t="inlineStr"/>
-      <c r="J1328" s="7" t="inlineStr"/>
+          <t>37:52</t>
+        </is>
+      </c>
+      <c r="I1328" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J1328" s="7" t="inlineStr">
+        <is>
+          <t>1. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1329">
       <c r="A1329" s="6" t="inlineStr">
@@ -66044,7 +66048,7 @@
       </c>
       <c r="D1329" s="7" t="inlineStr">
         <is>
-          <t>Kyrre Berland</t>
+          <t>Kristian Frøyen</t>
         </is>
       </c>
       <c r="E1329" s="6" t="inlineStr">
@@ -66064,19 +66068,11 @@
       </c>
       <c r="H1329" s="7" t="inlineStr">
         <is>
-          <t>1:19:33</t>
-        </is>
-      </c>
-      <c r="I1329" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J1329" s="7" t="inlineStr">
-        <is>
-          <t>1. plass</t>
-        </is>
-      </c>
+          <t>1:08:51</t>
+        </is>
+      </c>
+      <c r="I1329" s="7" t="inlineStr"/>
+      <c r="J1329" s="7" t="inlineStr"/>
     </row>
     <row r="1330">
       <c r="A1330" s="6" t="inlineStr">
@@ -66096,17 +66092,17 @@
       </c>
       <c r="D1330" s="7" t="inlineStr">
         <is>
-          <t>Catherine Vaugelade Pedersen</t>
+          <t>Kyrre Berland</t>
         </is>
       </c>
       <c r="E1330" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1330" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1330" s="6" t="inlineStr">
@@ -66116,17 +66112,17 @@
       </c>
       <c r="H1330" s="7" t="inlineStr">
         <is>
-          <t>1:24:05</t>
+          <t>1:19:33</t>
         </is>
       </c>
       <c r="I1330" s="7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J1330" s="7" t="inlineStr">
         <is>
-          <t>2. plass</t>
+          <t>1. plass</t>
         </is>
       </c>
     </row>
@@ -66148,7 +66144,7 @@
       </c>
       <c r="D1331" s="7" t="inlineStr">
         <is>
-          <t>Julie Thorp</t>
+          <t>Catherine Vaugelade Pedersen</t>
         </is>
       </c>
       <c r="E1331" s="6" t="inlineStr">
@@ -66168,11 +66164,19 @@
       </c>
       <c r="H1331" s="7" t="inlineStr">
         <is>
-          <t>1:24:21</t>
-        </is>
-      </c>
-      <c r="I1331" s="7" t="inlineStr"/>
-      <c r="J1331" s="7" t="inlineStr"/>
+          <t>1:24:05</t>
+        </is>
+      </c>
+      <c r="I1331" s="7" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="J1331" s="7" t="inlineStr">
+        <is>
+          <t>2. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1332">
       <c r="A1332" s="6" t="inlineStr">
@@ -66192,7 +66196,7 @@
       </c>
       <c r="D1332" s="7" t="inlineStr">
         <is>
-          <t>Janne Dahle</t>
+          <t>Julie Thorp</t>
         </is>
       </c>
       <c r="E1332" s="6" t="inlineStr">
@@ -66212,7 +66216,7 @@
       </c>
       <c r="H1332" s="7" t="inlineStr">
         <is>
-          <t>1:24:22</t>
+          <t>1:24:21</t>
         </is>
       </c>
       <c r="I1332" s="7" t="inlineStr"/>
@@ -66236,7 +66240,7 @@
       </c>
       <c r="D1333" s="7" t="inlineStr">
         <is>
-          <t>Sissel Oversand</t>
+          <t>Janne Dahle</t>
         </is>
       </c>
       <c r="E1333" s="6" t="inlineStr">
@@ -66256,7 +66260,7 @@
       </c>
       <c r="H1333" s="7" t="inlineStr">
         <is>
-          <t>1:30:27</t>
+          <t>1:24:22</t>
         </is>
       </c>
       <c r="I1333" s="7" t="inlineStr"/>
@@ -66280,7 +66284,7 @@
       </c>
       <c r="D1334" s="7" t="inlineStr">
         <is>
-          <t>Dong Zhang</t>
+          <t>Sissel Oversand</t>
         </is>
       </c>
       <c r="E1334" s="6" t="inlineStr">
@@ -66300,7 +66304,7 @@
       </c>
       <c r="H1334" s="7" t="inlineStr">
         <is>
-          <t>1:38:33</t>
+          <t>1:30:27</t>
         </is>
       </c>
       <c r="I1334" s="7" t="inlineStr"/>
@@ -66324,17 +66328,17 @@
       </c>
       <c r="D1335" s="7" t="inlineStr">
         <is>
-          <t>Christian Lillebo</t>
+          <t>Dong Zhang</t>
         </is>
       </c>
       <c r="E1335" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1335" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1335" s="6" t="inlineStr">
@@ -66344,7 +66348,7 @@
       </c>
       <c r="H1335" s="7" t="inlineStr">
         <is>
-          <t>1:41:11</t>
+          <t>1:38:33</t>
         </is>
       </c>
       <c r="I1335" s="7" t="inlineStr"/>
@@ -66368,7 +66372,7 @@
       </c>
       <c r="D1336" s="7" t="inlineStr">
         <is>
-          <t>Kristoffer Bugge</t>
+          <t>Christian Lillebo</t>
         </is>
       </c>
       <c r="E1336" s="6" t="inlineStr">
@@ -66383,12 +66387,12 @@
       </c>
       <c r="G1336" s="6" t="inlineStr">
         <is>
-          <t>Maraton</t>
+          <t>Halvmaraton</t>
         </is>
       </c>
       <c r="H1336" s="7" t="inlineStr">
         <is>
-          <t>2:45:23</t>
+          <t>1:41:11</t>
         </is>
       </c>
       <c r="I1336" s="7" t="inlineStr"/>
@@ -66412,17 +66416,17 @@
       </c>
       <c r="D1337" s="7" t="inlineStr">
         <is>
-          <t>Tone Gravvold</t>
+          <t>Kristoffer Bugge</t>
         </is>
       </c>
       <c r="E1337" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1337" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1337" s="6" t="inlineStr">
@@ -66432,7 +66436,7 @@
       </c>
       <c r="H1337" s="7" t="inlineStr">
         <is>
-          <t>3:36:52</t>
+          <t>2:45:23</t>
         </is>
       </c>
       <c r="I1337" s="7" t="inlineStr"/>
@@ -66456,7 +66460,7 @@
       </c>
       <c r="D1338" s="7" t="inlineStr">
         <is>
-          <t>Liv Berit Jegteberg Lystad</t>
+          <t>Tone Gravvold</t>
         </is>
       </c>
       <c r="E1338" s="6" t="inlineStr">
@@ -66476,7 +66480,7 @@
       </c>
       <c r="H1338" s="7" t="inlineStr">
         <is>
-          <t>4:20:11</t>
+          <t>3:36:52</t>
         </is>
       </c>
       <c r="I1338" s="7" t="inlineStr"/>
@@ -66495,12 +66499,12 @@
       </c>
       <c r="C1339" s="7" t="inlineStr">
         <is>
-          <t>Tyrvinglekene inn</t>
+          <t>Bislett Indoor Marathon</t>
         </is>
       </c>
       <c r="D1339" s="7" t="inlineStr">
         <is>
-          <t>Hanna Larsen</t>
+          <t>Liv Berit Jegteberg Lystad</t>
         </is>
       </c>
       <c r="E1339" s="6" t="inlineStr">
@@ -66515,24 +66519,16 @@
       </c>
       <c r="G1339" s="6" t="inlineStr">
         <is>
-          <t>800 m</t>
+          <t>Maraton</t>
         </is>
       </c>
       <c r="H1339" s="7" t="inlineStr">
         <is>
-          <t>2:10.21</t>
-        </is>
-      </c>
-      <c r="I1339" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J1339" s="7" t="inlineStr">
-        <is>
-          <t>1. plass</t>
-        </is>
-      </c>
+          <t>4:20:11</t>
+        </is>
+      </c>
+      <c r="I1339" s="7" t="inlineStr"/>
+      <c r="J1339" s="7" t="inlineStr"/>
     </row>
     <row r="1340">
       <c r="A1340" s="6" t="inlineStr">
@@ -66552,17 +66548,17 @@
       </c>
       <c r="D1340" s="7" t="inlineStr">
         <is>
-          <t>Noah Johannessen</t>
+          <t>Hanna Larsen</t>
         </is>
       </c>
       <c r="E1340" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1340" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1340" s="6" t="inlineStr">
@@ -66572,11 +66568,19 @@
       </c>
       <c r="H1340" s="7" t="inlineStr">
         <is>
-          <t>2:13.09</t>
-        </is>
-      </c>
-      <c r="I1340" s="7" t="inlineStr"/>
-      <c r="J1340" s="7" t="inlineStr"/>
+          <t>2:10.21</t>
+        </is>
+      </c>
+      <c r="I1340" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J1340" s="7" t="inlineStr">
+        <is>
+          <t>1. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1341">
       <c r="A1341" s="6" t="inlineStr">
@@ -66596,7 +66600,7 @@
       </c>
       <c r="D1341" s="7" t="inlineStr">
         <is>
-          <t>Theodor Berre Jacobsen</t>
+          <t>Noah Johannessen</t>
         </is>
       </c>
       <c r="E1341" s="6" t="inlineStr">
@@ -66611,12 +66615,12 @@
       </c>
       <c r="G1341" s="6" t="inlineStr">
         <is>
-          <t>3000 m</t>
+          <t>800 m</t>
         </is>
       </c>
       <c r="H1341" s="7" t="inlineStr">
         <is>
-          <t>8:25.71</t>
+          <t>2:13.09</t>
         </is>
       </c>
       <c r="I1341" s="7" t="inlineStr"/>
@@ -66640,7 +66644,7 @@
       </c>
       <c r="D1342" s="7" t="inlineStr">
         <is>
-          <t>Nicolay Andersen</t>
+          <t>Theodor Berre Jacobsen</t>
         </is>
       </c>
       <c r="E1342" s="6" t="inlineStr">
@@ -66660,7 +66664,7 @@
       </c>
       <c r="H1342" s="7" t="inlineStr">
         <is>
-          <t>8:26.64</t>
+          <t>8:25.71</t>
         </is>
       </c>
       <c r="I1342" s="7" t="inlineStr"/>
@@ -66684,7 +66688,7 @@
       </c>
       <c r="D1343" s="7" t="inlineStr">
         <is>
-          <t>Jakob Slengesol</t>
+          <t>Nicolay Andersen</t>
         </is>
       </c>
       <c r="E1343" s="6" t="inlineStr">
@@ -66704,15 +66708,11 @@
       </c>
       <c r="H1343" s="7" t="inlineStr">
         <is>
-          <t>9:26.53</t>
+          <t>8:26.64</t>
         </is>
       </c>
       <c r="I1343" s="7" t="inlineStr"/>
-      <c r="J1343" s="7" t="inlineStr">
-        <is>
-          <t>Offensiv åpning. Det kostet krefter mot slutten, men satsingen var der</t>
-        </is>
-      </c>
+      <c r="J1343" s="7" t="inlineStr"/>
     </row>
     <row r="1344">
       <c r="A1344" s="6" t="inlineStr">
@@ -66722,71 +66722,75 @@
       </c>
       <c r="B1344" s="6" t="inlineStr">
         <is>
-          <t>07.02.2026</t>
+          <t>08.02.2026</t>
         </is>
       </c>
       <c r="C1344" s="7" t="inlineStr">
         <is>
-          <t>Bislett Indoor Marathon</t>
+          <t>Tyrvinglekene inn</t>
         </is>
       </c>
       <c r="D1344" s="7" t="inlineStr">
         <is>
-          <t>Dory Kovacs</t>
+          <t>Jakob Slengesol</t>
         </is>
       </c>
       <c r="E1344" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1344" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1344" s="6" t="inlineStr">
         <is>
-          <t>Halvmaraton</t>
+          <t>3000 m</t>
         </is>
       </c>
       <c r="H1344" s="7" t="inlineStr">
         <is>
-          <t>1:28:13</t>
+          <t>9:26.53</t>
         </is>
       </c>
       <c r="I1344" s="7" t="inlineStr"/>
-      <c r="J1344" s="7" t="inlineStr"/>
+      <c r="J1344" s="7" t="inlineStr">
+        <is>
+          <t>Offensiv åpning. Det kostet krefter mot slutten, men satsingen var der</t>
+        </is>
+      </c>
     </row>
     <row r="1345">
       <c r="A1345" s="6" t="inlineStr">
         <is>
-          <t>Uke 5</t>
+          <t>Uke 6</t>
         </is>
       </c>
       <c r="B1345" s="6" t="inlineStr">
         <is>
-          <t>01.02.2026</t>
+          <t>07.02.2026</t>
         </is>
       </c>
       <c r="C1345" s="7" t="inlineStr">
         <is>
-          <t>Kagawa Marugame Half Marathon</t>
+          <t>Bislett Indoor Marathon</t>
         </is>
       </c>
       <c r="D1345" s="7" t="inlineStr">
         <is>
-          <t>Sondre Nordstad Moen</t>
+          <t>Dory Kovacs</t>
         </is>
       </c>
       <c r="E1345" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1345" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1345" s="6" t="inlineStr">
@@ -66796,7 +66800,7 @@
       </c>
       <c r="H1345" s="7" t="inlineStr">
         <is>
-          <t>1:00:46</t>
+          <t>1:28:13</t>
         </is>
       </c>
       <c r="I1345" s="7" t="inlineStr"/>
@@ -66815,12 +66819,12 @@
       </c>
       <c r="C1346" s="7" t="inlineStr">
         <is>
-          <t>Nordenkampen</t>
+          <t>Kagawa Marugame Half Marathon</t>
         </is>
       </c>
       <c r="D1346" s="7" t="inlineStr">
         <is>
-          <t>Sander Dybwad Mathiesen</t>
+          <t>Sondre Nordstad Moen</t>
         </is>
       </c>
       <c r="E1346" s="6" t="inlineStr">
@@ -66835,12 +66839,12 @@
       </c>
       <c r="G1346" s="6" t="inlineStr">
         <is>
-          <t>3000 m</t>
+          <t>Halvmaraton</t>
         </is>
       </c>
       <c r="H1346" s="7" t="inlineStr">
         <is>
-          <t>8:09.96</t>
+          <t>1:00:46</t>
         </is>
       </c>
       <c r="I1346" s="7" t="inlineStr"/>
@@ -66864,17 +66868,17 @@
       </c>
       <c r="D1347" s="7" t="inlineStr">
         <is>
-          <t>Madelène Wanvik Holum</t>
+          <t>Sander Dybwad Mathiesen</t>
         </is>
       </c>
       <c r="E1347" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1347" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1347" s="6" t="inlineStr">
@@ -66884,19 +66888,11 @@
       </c>
       <c r="H1347" s="7" t="inlineStr">
         <is>
-          <t>9:13.20</t>
-        </is>
-      </c>
-      <c r="I1347" s="7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="J1347" s="7" t="inlineStr">
-        <is>
-          <t>3. plass, innendørs PB</t>
-        </is>
-      </c>
+          <t>8:09.96</t>
+        </is>
+      </c>
+      <c r="I1347" s="7" t="inlineStr"/>
+      <c r="J1347" s="7" t="inlineStr"/>
     </row>
     <row r="1348">
       <c r="A1348" s="6" t="inlineStr">
@@ -66911,36 +66907,44 @@
       </c>
       <c r="C1348" s="7" t="inlineStr">
         <is>
-          <t>Winterrun Oslo</t>
+          <t>Nordenkampen</t>
         </is>
       </c>
       <c r="D1348" s="7" t="inlineStr">
         <is>
-          <t>Fredrik Camilo Halsbog</t>
+          <t>Madelène Wanvik Holum</t>
         </is>
       </c>
       <c r="E1348" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1348" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1348" s="6" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>3000 m</t>
         </is>
       </c>
       <c r="H1348" s="7" t="inlineStr">
         <is>
-          <t>19:47</t>
-        </is>
-      </c>
-      <c r="I1348" s="7" t="inlineStr"/>
-      <c r="J1348" s="7" t="inlineStr"/>
+          <t>9:13.20</t>
+        </is>
+      </c>
+      <c r="I1348" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J1348" s="7" t="inlineStr">
+        <is>
+          <t>3. plass, innendørs PB</t>
+        </is>
+      </c>
     </row>
     <row r="1349">
       <c r="A1349" s="6" t="inlineStr">
@@ -66960,39 +66964,31 @@
       </c>
       <c r="D1349" s="7" t="inlineStr">
         <is>
-          <t>Maria Bipop</t>
+          <t>Fredrik Camilo Halsbog</t>
         </is>
       </c>
       <c r="E1349" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1349" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1349" s="6" t="inlineStr">
         <is>
-          <t>10 km</t>
+          <t>5 km</t>
         </is>
       </c>
       <c r="H1349" s="7" t="inlineStr">
         <is>
-          <t>38:25</t>
-        </is>
-      </c>
-      <c r="I1349" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J1349" s="7" t="inlineStr">
-        <is>
-          <t>1. plass</t>
-        </is>
-      </c>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="I1349" s="7" t="inlineStr"/>
+      <c r="J1349" s="7" t="inlineStr"/>
     </row>
     <row r="1350">
       <c r="A1350" s="6" t="inlineStr">
@@ -67012,7 +67008,7 @@
       </c>
       <c r="D1350" s="7" t="inlineStr">
         <is>
-          <t>Sonia Nakamura Slettvåg (11 år)</t>
+          <t>Maria Bipop</t>
         </is>
       </c>
       <c r="E1350" s="6" t="inlineStr">
@@ -67032,11 +67028,19 @@
       </c>
       <c r="H1350" s="7" t="inlineStr">
         <is>
-          <t>48:00</t>
-        </is>
-      </c>
-      <c r="I1350" s="7" t="inlineStr"/>
-      <c r="J1350" s="7" t="inlineStr"/>
+          <t>38:25</t>
+        </is>
+      </c>
+      <c r="I1350" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J1350" s="7" t="inlineStr">
+        <is>
+          <t>1. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1351">
       <c r="A1351" s="6" t="inlineStr">
@@ -67056,7 +67060,7 @@
       </c>
       <c r="D1351" s="7" t="inlineStr">
         <is>
-          <t>Silje Solvang</t>
+          <t>Sonia Nakamura Slettvåg (11 år)</t>
         </is>
       </c>
       <c r="E1351" s="6" t="inlineStr">
@@ -67076,7 +67080,7 @@
       </c>
       <c r="H1351" s="7" t="inlineStr">
         <is>
-          <t>48:42</t>
+          <t>48:00</t>
         </is>
       </c>
       <c r="I1351" s="7" t="inlineStr"/>
@@ -67085,54 +67089,46 @@
     <row r="1352">
       <c r="A1352" s="6" t="inlineStr">
         <is>
-          <t>Uke 3</t>
+          <t>Uke 5</t>
         </is>
       </c>
       <c r="B1352" s="6" t="inlineStr">
         <is>
-          <t>18.01.2026</t>
+          <t>01.02.2026</t>
         </is>
       </c>
       <c r="C1352" s="7" t="inlineStr">
         <is>
-          <t>Bislett distanseserie 1 - 5K</t>
+          <t>Winterrun Oslo</t>
         </is>
       </c>
       <c r="D1352" s="7" t="inlineStr">
         <is>
-          <t>Kasper Sørlie-Reininger</t>
+          <t>Silje Solvang</t>
         </is>
       </c>
       <c r="E1352" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1352" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1352" s="6" t="inlineStr">
         <is>
-          <t>5 km</t>
+          <t>10 km</t>
         </is>
       </c>
       <c r="H1352" s="7" t="inlineStr">
         <is>
-          <t>15:07</t>
-        </is>
-      </c>
-      <c r="I1352" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J1352" s="7" t="inlineStr">
-        <is>
-          <t>1. plass, M18 19</t>
-        </is>
-      </c>
+          <t>48:42</t>
+        </is>
+      </c>
+      <c r="I1352" s="7" t="inlineStr"/>
+      <c r="J1352" s="7" t="inlineStr"/>
     </row>
     <row r="1353">
       <c r="A1353" s="6" t="inlineStr">
@@ -67152,7 +67148,7 @@
       </c>
       <c r="D1353" s="7" t="inlineStr">
         <is>
-          <t>Kristian Frøyen</t>
+          <t>Kasper Sørlie-Reininger</t>
         </is>
       </c>
       <c r="E1353" s="6" t="inlineStr">
@@ -67172,17 +67168,17 @@
       </c>
       <c r="H1353" s="7" t="inlineStr">
         <is>
-          <t>15:16</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="I1353" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="J1353" s="7" t="inlineStr">
         <is>
-          <t>3. plass</t>
+          <t>1. plass, M18 19</t>
         </is>
       </c>
     </row>
@@ -67204,7 +67200,7 @@
       </c>
       <c r="D1354" s="7" t="inlineStr">
         <is>
-          <t>Erik Rønneberg</t>
+          <t>Kristian Frøyen</t>
         </is>
       </c>
       <c r="E1354" s="6" t="inlineStr">
@@ -67224,11 +67220,19 @@
       </c>
       <c r="H1354" s="7" t="inlineStr">
         <is>
-          <t>15:17</t>
-        </is>
-      </c>
-      <c r="I1354" s="7" t="inlineStr"/>
-      <c r="J1354" s="7" t="inlineStr"/>
+          <t>15:16</t>
+        </is>
+      </c>
+      <c r="I1354" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J1354" s="7" t="inlineStr">
+        <is>
+          <t>3. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1355">
       <c r="A1355" s="6" t="inlineStr">
@@ -67248,7 +67252,7 @@
       </c>
       <c r="D1355" s="7" t="inlineStr">
         <is>
-          <t>Magnus Warvik</t>
+          <t>Erik Rønneberg</t>
         </is>
       </c>
       <c r="E1355" s="6" t="inlineStr">
@@ -67268,15 +67272,11 @@
       </c>
       <c r="H1355" s="7" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>15:17</t>
         </is>
       </c>
       <c r="I1355" s="7" t="inlineStr"/>
-      <c r="J1355" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1355" s="7" t="inlineStr"/>
     </row>
     <row r="1356">
       <c r="A1356" s="6" t="inlineStr">
@@ -67296,7 +67296,7 @@
       </c>
       <c r="D1356" s="7" t="inlineStr">
         <is>
-          <t>Fredrik Killerud</t>
+          <t>Magnus Warvik</t>
         </is>
       </c>
       <c r="E1356" s="6" t="inlineStr">
@@ -67316,11 +67316,15 @@
       </c>
       <c r="H1356" s="7" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="I1356" s="7" t="inlineStr"/>
-      <c r="J1356" s="7" t="inlineStr"/>
+      <c r="J1356" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1357">
       <c r="A1357" s="6" t="inlineStr">
@@ -67340,7 +67344,7 @@
       </c>
       <c r="D1357" s="7" t="inlineStr">
         <is>
-          <t>Thomas Kjellberg</t>
+          <t>Fredrik Killerud</t>
         </is>
       </c>
       <c r="E1357" s="6" t="inlineStr">
@@ -67360,7 +67364,7 @@
       </c>
       <c r="H1357" s="7" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="I1357" s="7" t="inlineStr"/>
@@ -67384,7 +67388,7 @@
       </c>
       <c r="D1358" s="7" t="inlineStr">
         <is>
-          <t>Martin Stray Egeberg</t>
+          <t>Thomas Kjellberg</t>
         </is>
       </c>
       <c r="E1358" s="6" t="inlineStr">
@@ -67404,7 +67408,7 @@
       </c>
       <c r="H1358" s="7" t="inlineStr">
         <is>
-          <t>15:33</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="I1358" s="7" t="inlineStr"/>
@@ -67428,7 +67432,7 @@
       </c>
       <c r="D1359" s="7" t="inlineStr">
         <is>
-          <t>Christoffer Hagen</t>
+          <t>Martin Stray Egeberg</t>
         </is>
       </c>
       <c r="E1359" s="6" t="inlineStr">
@@ -67448,7 +67452,7 @@
       </c>
       <c r="H1359" s="7" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:33</t>
         </is>
       </c>
       <c r="I1359" s="7" t="inlineStr"/>
@@ -67472,7 +67476,7 @@
       </c>
       <c r="D1360" s="7" t="inlineStr">
         <is>
-          <t>Truls Skarvøy</t>
+          <t>Christoffer Hagen</t>
         </is>
       </c>
       <c r="E1360" s="6" t="inlineStr">
@@ -67492,7 +67496,7 @@
       </c>
       <c r="H1360" s="7" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="I1360" s="7" t="inlineStr"/>
@@ -67516,17 +67520,17 @@
       </c>
       <c r="D1361" s="7" t="inlineStr">
         <is>
-          <t>Ine Bakken</t>
+          <t>Truls Skarvøy</t>
         </is>
       </c>
       <c r="E1361" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1361" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1361" s="6" t="inlineStr">
@@ -67536,19 +67540,11 @@
       </c>
       <c r="H1361" s="7" t="inlineStr">
         <is>
-          <t>16:31</t>
-        </is>
-      </c>
-      <c r="I1361" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J1361" s="7" t="inlineStr">
-        <is>
-          <t>1. plass</t>
-        </is>
-      </c>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="I1361" s="7" t="inlineStr"/>
+      <c r="J1361" s="7" t="inlineStr"/>
     </row>
     <row r="1362">
       <c r="A1362" s="6" t="inlineStr">
@@ -67568,17 +67564,17 @@
       </c>
       <c r="D1362" s="7" t="inlineStr">
         <is>
-          <t>Christian Lund Sørensen</t>
+          <t>Ine Bakken</t>
         </is>
       </c>
       <c r="E1362" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1362" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1362" s="6" t="inlineStr">
@@ -67588,11 +67584,19 @@
       </c>
       <c r="H1362" s="7" t="inlineStr">
         <is>
-          <t>16:35</t>
-        </is>
-      </c>
-      <c r="I1362" s="7" t="inlineStr"/>
-      <c r="J1362" s="7" t="inlineStr"/>
+          <t>16:31</t>
+        </is>
+      </c>
+      <c r="I1362" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J1362" s="7" t="inlineStr">
+        <is>
+          <t>1. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1363">
       <c r="A1363" s="6" t="inlineStr">
@@ -67612,7 +67616,7 @@
       </c>
       <c r="D1363" s="7" t="inlineStr">
         <is>
-          <t>Ruairí Long</t>
+          <t>Christian Lund Sørensen</t>
         </is>
       </c>
       <c r="E1363" s="6" t="inlineStr">
@@ -67632,15 +67636,11 @@
       </c>
       <c r="H1363" s="7" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="I1363" s="7" t="inlineStr"/>
-      <c r="J1363" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1363" s="7" t="inlineStr"/>
     </row>
     <row r="1364">
       <c r="A1364" s="6" t="inlineStr">
@@ -67660,7 +67660,7 @@
       </c>
       <c r="D1364" s="7" t="inlineStr">
         <is>
-          <t>Anton Heldal</t>
+          <t>Ruairí Long</t>
         </is>
       </c>
       <c r="E1364" s="6" t="inlineStr">
@@ -67680,11 +67680,15 @@
       </c>
       <c r="H1364" s="7" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="I1364" s="7" t="inlineStr"/>
-      <c r="J1364" s="7" t="inlineStr"/>
+      <c r="J1364" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1365">
       <c r="A1365" s="6" t="inlineStr">
@@ -67704,7 +67708,7 @@
       </c>
       <c r="D1365" s="7" t="inlineStr">
         <is>
-          <t>Anders Wigdahl</t>
+          <t>Anton Heldal</t>
         </is>
       </c>
       <c r="E1365" s="6" t="inlineStr">
@@ -67724,7 +67728,7 @@
       </c>
       <c r="H1365" s="7" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="I1365" s="7" t="inlineStr"/>
@@ -67748,7 +67752,7 @@
       </c>
       <c r="D1366" s="7" t="inlineStr">
         <is>
-          <t>Erlend Bruaset</t>
+          <t>Anders Wigdahl</t>
         </is>
       </c>
       <c r="E1366" s="6" t="inlineStr">
@@ -67768,7 +67772,7 @@
       </c>
       <c r="H1366" s="7" t="inlineStr">
         <is>
-          <t>17:44</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="I1366" s="7" t="inlineStr"/>
@@ -67792,7 +67796,7 @@
       </c>
       <c r="D1367" s="7" t="inlineStr">
         <is>
-          <t>Ole Kristian Gjertsen</t>
+          <t>Erlend Bruaset</t>
         </is>
       </c>
       <c r="E1367" s="6" t="inlineStr">
@@ -67812,15 +67816,11 @@
       </c>
       <c r="H1367" s="7" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:44</t>
         </is>
       </c>
       <c r="I1367" s="7" t="inlineStr"/>
-      <c r="J1367" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1367" s="7" t="inlineStr"/>
     </row>
     <row r="1368">
       <c r="A1368" s="6" t="inlineStr">
@@ -67840,17 +67840,17 @@
       </c>
       <c r="D1368" s="7" t="inlineStr">
         <is>
-          <t>Marte Sønstevold</t>
+          <t>Ole Kristian Gjertsen</t>
         </is>
       </c>
       <c r="E1368" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1368" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1368" s="6" t="inlineStr">
@@ -67860,11 +67860,15 @@
       </c>
       <c r="H1368" s="7" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="I1368" s="7" t="inlineStr"/>
-      <c r="J1368" s="7" t="inlineStr"/>
+      <c r="J1368" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1369">
       <c r="A1369" s="6" t="inlineStr">
@@ -67884,7 +67888,7 @@
       </c>
       <c r="D1369" s="7" t="inlineStr">
         <is>
-          <t>Henriette Sæterdal Semb</t>
+          <t>Marte Sønstevold</t>
         </is>
       </c>
       <c r="E1369" s="6" t="inlineStr">
@@ -67904,7 +67908,7 @@
       </c>
       <c r="H1369" s="7" t="inlineStr">
         <is>
-          <t>18:06</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="I1369" s="7" t="inlineStr"/>
@@ -67928,7 +67932,7 @@
       </c>
       <c r="D1370" s="7" t="inlineStr">
         <is>
-          <t>Rebekka Haugland</t>
+          <t>Henriette Sæterdal Semb</t>
         </is>
       </c>
       <c r="E1370" s="6" t="inlineStr">
@@ -67948,7 +67952,7 @@
       </c>
       <c r="H1370" s="7" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:06</t>
         </is>
       </c>
       <c r="I1370" s="7" t="inlineStr"/>
@@ -67972,7 +67976,7 @@
       </c>
       <c r="D1371" s="7" t="inlineStr">
         <is>
-          <t>Catherine Vaugelade Pedersen</t>
+          <t>Rebekka Haugland</t>
         </is>
       </c>
       <c r="E1371" s="6" t="inlineStr">
@@ -67992,7 +67996,7 @@
       </c>
       <c r="H1371" s="7" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="I1371" s="7" t="inlineStr"/>
@@ -68016,7 +68020,7 @@
       </c>
       <c r="D1372" s="7" t="inlineStr">
         <is>
-          <t>Kara Meunier</t>
+          <t>Catherine Vaugelade Pedersen</t>
         </is>
       </c>
       <c r="E1372" s="6" t="inlineStr">
@@ -68036,7 +68040,7 @@
       </c>
       <c r="H1372" s="7" t="inlineStr">
         <is>
-          <t>18:16</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="I1372" s="7" t="inlineStr"/>
@@ -68060,17 +68064,17 @@
       </c>
       <c r="D1373" s="7" t="inlineStr">
         <is>
-          <t>Ole Jonas Nybø</t>
+          <t>Kara Meunier</t>
         </is>
       </c>
       <c r="E1373" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1373" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1373" s="6" t="inlineStr">
@@ -68080,7 +68084,7 @@
       </c>
       <c r="H1373" s="7" t="inlineStr">
         <is>
-          <t>18:29</t>
+          <t>18:16</t>
         </is>
       </c>
       <c r="I1373" s="7" t="inlineStr"/>
@@ -68104,7 +68108,7 @@
       </c>
       <c r="D1374" s="7" t="inlineStr">
         <is>
-          <t>Nicolai Borenstein</t>
+          <t>Ole Jonas Nybø</t>
         </is>
       </c>
       <c r="E1374" s="6" t="inlineStr">
@@ -68124,7 +68128,7 @@
       </c>
       <c r="H1374" s="7" t="inlineStr">
         <is>
-          <t>18:46</t>
+          <t>18:29</t>
         </is>
       </c>
       <c r="I1374" s="7" t="inlineStr"/>
@@ -68148,7 +68152,7 @@
       </c>
       <c r="D1375" s="7" t="inlineStr">
         <is>
-          <t>Fredrik Camilo Halsbog</t>
+          <t>Nicolai Borenstein</t>
         </is>
       </c>
       <c r="E1375" s="6" t="inlineStr">
@@ -68168,15 +68172,11 @@
       </c>
       <c r="H1375" s="7" t="inlineStr">
         <is>
-          <t>18:54</t>
+          <t>18:46</t>
         </is>
       </c>
       <c r="I1375" s="7" t="inlineStr"/>
-      <c r="J1375" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1375" s="7" t="inlineStr"/>
     </row>
     <row r="1376">
       <c r="A1376" s="6" t="inlineStr">
@@ -68196,7 +68196,7 @@
       </c>
       <c r="D1376" s="7" t="inlineStr">
         <is>
-          <t>Runar Oesthaug</t>
+          <t>Fredrik Camilo Halsbog</t>
         </is>
       </c>
       <c r="E1376" s="6" t="inlineStr">
@@ -68216,11 +68216,15 @@
       </c>
       <c r="H1376" s="7" t="inlineStr">
         <is>
-          <t>18:56</t>
+          <t>18:54</t>
         </is>
       </c>
       <c r="I1376" s="7" t="inlineStr"/>
-      <c r="J1376" s="7" t="inlineStr"/>
+      <c r="J1376" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1377">
       <c r="A1377" s="6" t="inlineStr">
@@ -68240,7 +68244,7 @@
       </c>
       <c r="D1377" s="7" t="inlineStr">
         <is>
-          <t>Kjetil Aakvik</t>
+          <t>Runar Oesthaug</t>
         </is>
       </c>
       <c r="E1377" s="6" t="inlineStr">
@@ -68260,7 +68264,7 @@
       </c>
       <c r="H1377" s="7" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:56</t>
         </is>
       </c>
       <c r="I1377" s="7" t="inlineStr"/>
@@ -68284,7 +68288,7 @@
       </c>
       <c r="D1378" s="7" t="inlineStr">
         <is>
-          <t>Simen Hagerup Kjeldsen</t>
+          <t>Kjetil Aakvik</t>
         </is>
       </c>
       <c r="E1378" s="6" t="inlineStr">
@@ -68304,7 +68308,7 @@
       </c>
       <c r="H1378" s="7" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="I1378" s="7" t="inlineStr"/>
@@ -68328,17 +68332,17 @@
       </c>
       <c r="D1379" s="7" t="inlineStr">
         <is>
-          <t>Sofie</t>
+          <t>Simen Hagerup Kjeldsen</t>
         </is>
       </c>
       <c r="E1379" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1379" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1379" s="6" t="inlineStr">
@@ -68348,7 +68352,7 @@
       </c>
       <c r="H1379" s="7" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="I1379" s="7" t="inlineStr"/>
@@ -68372,7 +68376,7 @@
       </c>
       <c r="D1380" s="7" t="inlineStr">
         <is>
-          <t>Julie Lous</t>
+          <t>Sofie</t>
         </is>
       </c>
       <c r="E1380" s="6" t="inlineStr">
@@ -68392,7 +68396,7 @@
       </c>
       <c r="H1380" s="7" t="inlineStr">
         <is>
-          <t>19:32</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="I1380" s="7" t="inlineStr"/>
@@ -68416,7 +68420,7 @@
       </c>
       <c r="D1381" s="7" t="inlineStr">
         <is>
-          <t>Torill Ytterhus Haugset</t>
+          <t>Julie Lous</t>
         </is>
       </c>
       <c r="E1381" s="6" t="inlineStr">
@@ -68436,7 +68440,7 @@
       </c>
       <c r="H1381" s="7" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:32</t>
         </is>
       </c>
       <c r="I1381" s="7" t="inlineStr"/>
@@ -68460,17 +68464,17 @@
       </c>
       <c r="D1382" s="7" t="inlineStr">
         <is>
-          <t>Ole Anders</t>
+          <t>Torill Ytterhus Haugset</t>
         </is>
       </c>
       <c r="E1382" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1382" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1382" s="6" t="inlineStr">
@@ -68480,15 +68484,11 @@
       </c>
       <c r="H1382" s="7" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="I1382" s="7" t="inlineStr"/>
-      <c r="J1382" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1382" s="7" t="inlineStr"/>
     </row>
     <row r="1383">
       <c r="A1383" s="6" t="inlineStr">
@@ -68508,17 +68508,17 @@
       </c>
       <c r="D1383" s="7" t="inlineStr">
         <is>
-          <t>Siri Hegsvold</t>
+          <t>Ole Anders</t>
         </is>
       </c>
       <c r="E1383" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1383" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1383" s="6" t="inlineStr">
@@ -68528,11 +68528,15 @@
       </c>
       <c r="H1383" s="7" t="inlineStr">
         <is>
-          <t>20:24</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="I1383" s="7" t="inlineStr"/>
-      <c r="J1383" s="7" t="inlineStr"/>
+      <c r="J1383" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1384">
       <c r="A1384" s="6" t="inlineStr">
@@ -68552,7 +68556,7 @@
       </c>
       <c r="D1384" s="7" t="inlineStr">
         <is>
-          <t>Tone Gravvold</t>
+          <t>Siri Hegsvold</t>
         </is>
       </c>
       <c r="E1384" s="6" t="inlineStr">
@@ -68572,15 +68576,11 @@
       </c>
       <c r="H1384" s="7" t="inlineStr">
         <is>
-          <t>20:30</t>
+          <t>20:24</t>
         </is>
       </c>
       <c r="I1384" s="7" t="inlineStr"/>
-      <c r="J1384" s="7" t="inlineStr">
-        <is>
-          <t>para</t>
-        </is>
-      </c>
+      <c r="J1384" s="7" t="inlineStr"/>
     </row>
     <row r="1385">
       <c r="A1385" s="6" t="inlineStr">
@@ -68600,7 +68600,7 @@
       </c>
       <c r="D1385" s="7" t="inlineStr">
         <is>
-          <t>Ingrid Skomedal Klovning</t>
+          <t>Tone Gravvold</t>
         </is>
       </c>
       <c r="E1385" s="6" t="inlineStr">
@@ -68620,11 +68620,15 @@
       </c>
       <c r="H1385" s="7" t="inlineStr">
         <is>
-          <t>20:33</t>
+          <t>20:30</t>
         </is>
       </c>
       <c r="I1385" s="7" t="inlineStr"/>
-      <c r="J1385" s="7" t="inlineStr"/>
+      <c r="J1385" s="7" t="inlineStr">
+        <is>
+          <t>para</t>
+        </is>
+      </c>
     </row>
     <row r="1386">
       <c r="A1386" s="6" t="inlineStr">
@@ -68644,17 +68648,17 @@
       </c>
       <c r="D1386" s="7" t="inlineStr">
         <is>
-          <t>Magnus Warvik</t>
+          <t>Ingrid Skomedal Klovning</t>
         </is>
       </c>
       <c r="E1386" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1386" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1386" s="6" t="inlineStr">
@@ -68668,11 +68672,7 @@
         </is>
       </c>
       <c r="I1386" s="7" t="inlineStr"/>
-      <c r="J1386" s="7" t="inlineStr">
-        <is>
-          <t>fartsholder</t>
-        </is>
-      </c>
+      <c r="J1386" s="7" t="inlineStr"/>
     </row>
     <row r="1387">
       <c r="A1387" s="6" t="inlineStr">
@@ -68692,17 +68692,17 @@
       </c>
       <c r="D1387" s="7" t="inlineStr">
         <is>
-          <t>Michael Floater</t>
+          <t>Magnus Warvik</t>
         </is>
       </c>
       <c r="E1387" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1387" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1387" s="6" t="inlineStr">
@@ -68712,11 +68712,15 @@
       </c>
       <c r="H1387" s="7" t="inlineStr">
         <is>
-          <t>21:06</t>
+          <t>20:33</t>
         </is>
       </c>
       <c r="I1387" s="7" t="inlineStr"/>
-      <c r="J1387" s="7" t="inlineStr"/>
+      <c r="J1387" s="7" t="inlineStr">
+        <is>
+          <t>fartsholder</t>
+        </is>
+      </c>
     </row>
     <row r="1388">
       <c r="A1388" s="6" t="inlineStr">
@@ -68736,7 +68740,7 @@
       </c>
       <c r="D1388" s="7" t="inlineStr">
         <is>
-          <t>Sonia Slettvåg</t>
+          <t>Michael Floater</t>
         </is>
       </c>
       <c r="E1388" s="6" t="inlineStr">
@@ -68756,15 +68760,11 @@
       </c>
       <c r="H1388" s="7" t="inlineStr">
         <is>
-          <t>21:39</t>
+          <t>21:06</t>
         </is>
       </c>
       <c r="I1388" s="7" t="inlineStr"/>
-      <c r="J1388" s="7" t="inlineStr">
-        <is>
-          <t>K11</t>
-        </is>
-      </c>
+      <c r="J1388" s="7" t="inlineStr"/>
     </row>
     <row r="1389">
       <c r="A1389" s="6" t="inlineStr">
@@ -68784,7 +68784,7 @@
       </c>
       <c r="D1389" s="7" t="inlineStr">
         <is>
-          <t>Ida Matre</t>
+          <t>Sonia Slettvåg</t>
         </is>
       </c>
       <c r="E1389" s="6" t="inlineStr">
@@ -68804,11 +68804,15 @@
       </c>
       <c r="H1389" s="7" t="inlineStr">
         <is>
-          <t>21:40</t>
+          <t>21:39</t>
         </is>
       </c>
       <c r="I1389" s="7" t="inlineStr"/>
-      <c r="J1389" s="7" t="inlineStr"/>
+      <c r="J1389" s="7" t="inlineStr">
+        <is>
+          <t>K11</t>
+        </is>
+      </c>
     </row>
     <row r="1390">
       <c r="A1390" s="6" t="inlineStr">
@@ -68828,7 +68832,7 @@
       </c>
       <c r="D1390" s="7" t="inlineStr">
         <is>
-          <t>Róisín Long</t>
+          <t>Ida Matre</t>
         </is>
       </c>
       <c r="E1390" s="6" t="inlineStr">
@@ -68848,7 +68852,7 @@
       </c>
       <c r="H1390" s="7" t="inlineStr">
         <is>
-          <t>21:43</t>
+          <t>21:40</t>
         </is>
       </c>
       <c r="I1390" s="7" t="inlineStr"/>
@@ -68872,7 +68876,7 @@
       </c>
       <c r="D1391" s="7" t="inlineStr">
         <is>
-          <t>June Kieu-Van Thi Bui</t>
+          <t>Róisín Long</t>
         </is>
       </c>
       <c r="E1391" s="6" t="inlineStr">
@@ -68892,7 +68896,7 @@
       </c>
       <c r="H1391" s="7" t="inlineStr">
         <is>
-          <t>21:48</t>
+          <t>21:43</t>
         </is>
       </c>
       <c r="I1391" s="7" t="inlineStr"/>
@@ -68916,17 +68920,17 @@
       </c>
       <c r="D1392" s="7" t="inlineStr">
         <is>
-          <t>Christian Lillebo</t>
+          <t>June Kieu-Van Thi Bui</t>
         </is>
       </c>
       <c r="E1392" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1392" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1392" s="6" t="inlineStr">
@@ -68936,7 +68940,7 @@
       </c>
       <c r="H1392" s="7" t="inlineStr">
         <is>
-          <t>22:23</t>
+          <t>21:48</t>
         </is>
       </c>
       <c r="I1392" s="7" t="inlineStr"/>
@@ -68960,17 +68964,17 @@
       </c>
       <c r="D1393" s="7" t="inlineStr">
         <is>
-          <t>Marie Reimer</t>
+          <t>Christian Lillebo</t>
         </is>
       </c>
       <c r="E1393" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1393" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1393" s="6" t="inlineStr">
@@ -68980,7 +68984,7 @@
       </c>
       <c r="H1393" s="7" t="inlineStr">
         <is>
-          <t>23:28</t>
+          <t>22:23</t>
         </is>
       </c>
       <c r="I1393" s="7" t="inlineStr"/>
@@ -69004,7 +69008,7 @@
       </c>
       <c r="D1394" s="7" t="inlineStr">
         <is>
-          <t>Ernst Herlof Kristiansen</t>
+          <t>Marie Reimer</t>
         </is>
       </c>
       <c r="E1394" s="6" t="inlineStr">
@@ -69024,15 +69028,11 @@
       </c>
       <c r="H1394" s="7" t="inlineStr">
         <is>
-          <t>25:17</t>
+          <t>23:28</t>
         </is>
       </c>
       <c r="I1394" s="7" t="inlineStr"/>
-      <c r="J1394" s="7" t="inlineStr">
-        <is>
-          <t>M75-79</t>
-        </is>
-      </c>
+      <c r="J1394" s="7" t="inlineStr"/>
     </row>
     <row r="1395">
       <c r="A1395" s="6" t="inlineStr">
@@ -69047,38 +69047,38 @@
       </c>
       <c r="C1395" s="7" t="inlineStr">
         <is>
-          <t>Sandsjöbacka Trail 2026</t>
+          <t>Bislett distanseserie 1 - 5K</t>
         </is>
       </c>
       <c r="D1395" s="7" t="inlineStr">
         <is>
-          <t>Askild Vatnbakk Larsen</t>
+          <t>Ernst Herlof Kristiansen</t>
         </is>
       </c>
       <c r="E1395" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1395" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1395" s="6" t="inlineStr">
         <is>
-          <t>30 km</t>
-        </is>
-      </c>
-      <c r="H1395" s="7" t="inlineStr"/>
-      <c r="I1395" s="7" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
+          <t>5 km</t>
+        </is>
+      </c>
+      <c r="H1395" s="7" t="inlineStr">
+        <is>
+          <t>25:17</t>
+        </is>
+      </c>
+      <c r="I1395" s="7" t="inlineStr"/>
       <c r="J1395" s="7" t="inlineStr">
         <is>
-          <t>2. plass</t>
+          <t>M75-79</t>
         </is>
       </c>
     </row>
@@ -69100,7 +69100,7 @@
       </c>
       <c r="D1396" s="7" t="inlineStr">
         <is>
-          <t>Kristoffer Eftedal</t>
+          <t>Askild Vatnbakk Larsen</t>
         </is>
       </c>
       <c r="E1396" s="6" t="inlineStr">
@@ -69121,12 +69121,12 @@
       <c r="H1396" s="7" t="inlineStr"/>
       <c r="I1396" s="7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="J1396" s="7" t="inlineStr">
         <is>
-          <t>3. plass</t>
+          <t>2. plass</t>
         </is>
       </c>
     </row>
@@ -69148,7 +69148,7 @@
       </c>
       <c r="D1397" s="7" t="inlineStr">
         <is>
-          <t>Steffen Brufladt</t>
+          <t>Kristoffer Eftedal</t>
         </is>
       </c>
       <c r="E1397" s="6" t="inlineStr">
@@ -69169,10 +69169,14 @@
       <c r="H1397" s="7" t="inlineStr"/>
       <c r="I1397" s="7" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="J1397" s="7" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="J1397" s="7" t="inlineStr">
+        <is>
+          <t>3. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1398">
       <c r="A1398" s="6" t="inlineStr">
@@ -69192,35 +69196,31 @@
       </c>
       <c r="D1398" s="7" t="inlineStr">
         <is>
-          <t>Maria Bipop</t>
+          <t>Steffen Brufladt</t>
         </is>
       </c>
       <c r="E1398" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1398" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1398" s="6" t="inlineStr">
         <is>
-          <t>60 km</t>
+          <t>30 km</t>
         </is>
       </c>
       <c r="H1398" s="7" t="inlineStr"/>
       <c r="I1398" s="7" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="J1398" s="7" t="inlineStr">
-        <is>
-          <t>1. plass</t>
-        </is>
-      </c>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="J1398" s="7" t="inlineStr"/>
     </row>
     <row r="1399">
       <c r="A1399" s="6" t="inlineStr">
@@ -69235,36 +69235,40 @@
       </c>
       <c r="C1399" s="7" t="inlineStr">
         <is>
-          <t>Santa Pola Halvmaraton</t>
+          <t>Sandsjöbacka Trail 2026</t>
         </is>
       </c>
       <c r="D1399" s="7" t="inlineStr">
         <is>
-          <t>Simon Skretting</t>
+          <t>Maria Bipop</t>
         </is>
       </c>
       <c r="E1399" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1399" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1399" s="6" t="inlineStr">
         <is>
-          <t>Halvmaraton</t>
-        </is>
-      </c>
-      <c r="H1399" s="7" t="inlineStr">
-        <is>
-          <t>1:15:18</t>
-        </is>
-      </c>
-      <c r="I1399" s="7" t="inlineStr"/>
-      <c r="J1399" s="7" t="inlineStr"/>
+          <t>60 km</t>
+        </is>
+      </c>
+      <c r="H1399" s="7" t="inlineStr"/>
+      <c r="I1399" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="J1399" s="7" t="inlineStr">
+        <is>
+          <t>1. plass</t>
+        </is>
+      </c>
     </row>
     <row r="1400">
       <c r="A1400" s="6" t="inlineStr">
@@ -69284,7 +69288,7 @@
       </c>
       <c r="D1400" s="7" t="inlineStr">
         <is>
-          <t>Pål Erik</t>
+          <t>Simon Skretting</t>
         </is>
       </c>
       <c r="E1400" s="6" t="inlineStr">
@@ -69304,7 +69308,7 @@
       </c>
       <c r="H1400" s="7" t="inlineStr">
         <is>
-          <t>1:16:57</t>
+          <t>1:15:18</t>
         </is>
       </c>
       <c r="I1400" s="7" t="inlineStr"/>
@@ -69313,42 +69317,42 @@
     <row r="1401">
       <c r="A1401" s="6" t="inlineStr">
         <is>
-          <t>Uke 2</t>
+          <t>Uke 3</t>
         </is>
       </c>
       <c r="B1401" s="6" t="inlineStr">
         <is>
-          <t>11.01.2026</t>
+          <t>18.01.2026</t>
         </is>
       </c>
       <c r="C1401" s="7" t="inlineStr">
         <is>
-          <t>Hoka Solastranden 10k</t>
+          <t>Santa Pola Halvmaraton</t>
         </is>
       </c>
       <c r="D1401" s="7" t="inlineStr">
         <is>
-          <t>Marie Bringsvor</t>
+          <t>Pål Erik</t>
         </is>
       </c>
       <c r="E1401" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1401" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1401" s="6" t="inlineStr">
         <is>
-          <t>10 km</t>
+          <t>Halvmaraton</t>
         </is>
       </c>
       <c r="H1401" s="7" t="inlineStr">
         <is>
-          <t>39:41</t>
+          <t>1:16:57</t>
         </is>
       </c>
       <c r="I1401" s="7" t="inlineStr"/>
@@ -69367,22 +69371,22 @@
       </c>
       <c r="C1402" s="7" t="inlineStr">
         <is>
-          <t>Valencia 10k</t>
+          <t>Hoka Solastranden 10k</t>
         </is>
       </c>
       <c r="D1402" s="7" t="inlineStr">
         <is>
-          <t>Trond Einar Moen Pedersli</t>
+          <t>Marie Bringsvor</t>
         </is>
       </c>
       <c r="E1402" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1402" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1402" s="6" t="inlineStr">
@@ -69392,7 +69396,7 @@
       </c>
       <c r="H1402" s="7" t="inlineStr">
         <is>
-          <t>29:52</t>
+          <t>39:41</t>
         </is>
       </c>
       <c r="I1402" s="7" t="inlineStr"/>
@@ -69416,7 +69420,7 @@
       </c>
       <c r="D1403" s="7" t="inlineStr">
         <is>
-          <t>Simon Skretting</t>
+          <t>Trond Einar Moen Pedersli</t>
         </is>
       </c>
       <c r="E1403" s="6" t="inlineStr">
@@ -69436,7 +69440,7 @@
       </c>
       <c r="H1403" s="7" t="inlineStr">
         <is>
-          <t>33:48</t>
+          <t>29:52</t>
         </is>
       </c>
       <c r="I1403" s="7" t="inlineStr"/>
@@ -69460,7 +69464,7 @@
       </c>
       <c r="D1404" s="7" t="inlineStr">
         <is>
-          <t>Henrik Victor Hansen</t>
+          <t>Simon Skretting</t>
         </is>
       </c>
       <c r="E1404" s="6" t="inlineStr">
@@ -69480,7 +69484,7 @@
       </c>
       <c r="H1404" s="7" t="inlineStr">
         <is>
-          <t>34:46</t>
+          <t>33:48</t>
         </is>
       </c>
       <c r="I1404" s="7" t="inlineStr"/>
@@ -69504,17 +69508,17 @@
       </c>
       <c r="D1405" s="7" t="inlineStr">
         <is>
-          <t>Ingrid Helene Nyhus</t>
+          <t>Henrik Victor Hansen</t>
         </is>
       </c>
       <c r="E1405" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1405" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1405" s="6" t="inlineStr">
@@ -69524,7 +69528,7 @@
       </c>
       <c r="H1405" s="7" t="inlineStr">
         <is>
-          <t>35:09</t>
+          <t>34:46</t>
         </is>
       </c>
       <c r="I1405" s="7" t="inlineStr"/>
@@ -69548,17 +69552,17 @@
       </c>
       <c r="D1406" s="7" t="inlineStr">
         <is>
-          <t>Nicolai Lujan Foss</t>
+          <t>Ingrid Helene Nyhus</t>
         </is>
       </c>
       <c r="E1406" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1406" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1406" s="6" t="inlineStr">
@@ -69568,7 +69572,7 @@
       </c>
       <c r="H1406" s="7" t="inlineStr">
         <is>
-          <t>35:40</t>
+          <t>35:09</t>
         </is>
       </c>
       <c r="I1406" s="7" t="inlineStr"/>
@@ -69592,17 +69596,17 @@
       </c>
       <c r="D1407" s="7" t="inlineStr">
         <is>
-          <t>Hanna Larsen</t>
+          <t>Nicolai Lujan Foss</t>
         </is>
       </c>
       <c r="E1407" s="6" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>M</t>
         </is>
       </c>
       <c r="F1407" s="6" t="inlineStr">
         <is>
-          <t>K åpen</t>
+          <t>M åpen</t>
         </is>
       </c>
       <c r="G1407" s="6" t="inlineStr">
@@ -69612,7 +69616,7 @@
       </c>
       <c r="H1407" s="7" t="inlineStr">
         <is>
-          <t>36:09</t>
+          <t>35:40</t>
         </is>
       </c>
       <c r="I1407" s="7" t="inlineStr"/>
@@ -69636,17 +69640,17 @@
       </c>
       <c r="D1408" s="7" t="inlineStr">
         <is>
-          <t>Jakov Semaskevic</t>
+          <t>Hanna Larsen</t>
         </is>
       </c>
       <c r="E1408" s="6" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>K</t>
         </is>
       </c>
       <c r="F1408" s="6" t="inlineStr">
         <is>
-          <t>M åpen</t>
+          <t>K åpen</t>
         </is>
       </c>
       <c r="G1408" s="6" t="inlineStr">
@@ -69656,7 +69660,7 @@
       </c>
       <c r="H1408" s="7" t="inlineStr">
         <is>
-          <t>36:10</t>
+          <t>36:09</t>
         </is>
       </c>
       <c r="I1408" s="7" t="inlineStr"/>
@@ -69680,35 +69684,79 @@
       </c>
       <c r="D1409" s="7" t="inlineStr">
         <is>
+          <t>Jakov Semaskevic</t>
+        </is>
+      </c>
+      <c r="E1409" s="6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="F1409" s="6" t="inlineStr">
+        <is>
+          <t>M åpen</t>
+        </is>
+      </c>
+      <c r="G1409" s="6" t="inlineStr">
+        <is>
+          <t>10 km</t>
+        </is>
+      </c>
+      <c r="H1409" s="7" t="inlineStr">
+        <is>
+          <t>36:10</t>
+        </is>
+      </c>
+      <c r="I1409" s="7" t="inlineStr"/>
+      <c r="J1409" s="7" t="inlineStr"/>
+    </row>
+    <row r="1410">
+      <c r="A1410" s="6" t="inlineStr">
+        <is>
+          <t>Uke 2</t>
+        </is>
+      </c>
+      <c r="B1410" s="6" t="inlineStr">
+        <is>
+          <t>11.01.2026</t>
+        </is>
+      </c>
+      <c r="C1410" s="7" t="inlineStr">
+        <is>
+          <t>Valencia 10k</t>
+        </is>
+      </c>
+      <c r="D1410" s="7" t="inlineStr">
+        <is>
           <t>Synøve Brox</t>
         </is>
       </c>
-      <c r="E1409" s="6" t="inlineStr">
+      <c r="E1410" s="6" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="F1409" s="6" t="inlineStr">
+      <c r="F1410" s="6" t="inlineStr">
         <is>
           <t>K åpen</t>
         </is>
       </c>
-      <c r="G1409" s="6" t="inlineStr">
+      <c r="G1410" s="6" t="inlineStr">
         <is>
           <t>10 km</t>
         </is>
       </c>
-      <c r="H1409" s="7" t="inlineStr">
+      <c r="H1410" s="7" t="inlineStr">
         <is>
           <t>40:33</t>
         </is>
       </c>
-      <c r="I1409" s="7" t="inlineStr">
+      <c r="I1410" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="J1409" s="7" t="inlineStr">
+      <c r="J1410" s="7" t="inlineStr">
         <is>
           <t>Vinner av F65-klassen, 1. plass</t>
         </is>
@@ -70306,14 +70354,14 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Castellon 10k</t>
+          <t>Castellon 10k, New Delhi Half Marathon 2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix security scan findings and harden publishing
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -1710,7 +1710,7 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>NM terrengultra; 2. kvinne; totalplass 13; aldersklasseplass 1; 50 km etter 8 t 40 min 21 sek; forvarsling etter 12 t 01 min 45 sek</t>
+          <t>NM terrengultra; 2; kvinne; totalplass 13; aldersklasseplass 1; 50 km etter 8 t 40 min 21 sek; forvarsling etter 12 t 01 min 45 sek</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>6. kvinne, motbakke</t>
+          <t>6; kvinne, motbakke</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1958,7 @@
       <c r="I34" s="7" t="inlineStr"/>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>Oordegem, Belgia; plassering ikke publisert etter brukerens instruks</t>
+          <t>Oordegem, Belgia</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2006,7 @@
       <c r="I35" s="7" t="inlineStr"/>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>Oordegem, Belgia; plassering ikke publisert etter brukerens instruks</t>
+          <t>Oordegem, Belgia</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       <c r="I36" s="7" t="inlineStr"/>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>Oordegem, Belgia; plassering ikke publisert etter brukerens instruks</t>
+          <t>Oordegem, Belgia</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>Tusser 24 km; terrengløp; 10. mann; totalplass 12; M15-19 klasse 1; kontrollpunkt 2 t 44 min 09 sek; siste 1 min 25 sek</t>
+          <t>Tusser 24 km; terrengløp; 10; mann; totalplass 12; M15-19 klasse 1; kontrollpunkt 2 t 44 min 09 sek; siste 1 min 25 sek</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne; 4600 hm; Four Summits</t>
+          <t>1; kvinne; 4600 hm; Four Summits</t>
         </is>
       </c>
     </row>
@@ -2210,7 +2210,7 @@
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>terrengløp; 1. kvinne; totalplass 3; Tänndalen, Sverige</t>
+          <t>terrengløp; 1; kvinne; totalplass 3; Tänndalen, Sverige</t>
         </is>
       </c>
     </row>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne; totalplass 16; K65-69 klasse 1</t>
+          <t>3; kvinne; totalplass 16; K65-69 klasse 1</t>
         </is>
       </c>
     </row>
@@ -2314,7 +2314,7 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>1. mann; finale; Heat 2</t>
+          <t>1; mann; finale; Heat 2</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>11. mann; finale; Heat 2</t>
+          <t>11; mann; finale; Heat 2</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>13. mann; finale; Heat 2; PB</t>
+          <t>13; mann; finale; Heat 2; PB</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>14. mann; finale; Heat 2; PB</t>
+          <t>14; mann; finale; Heat 2; PB</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne; finale</t>
+          <t>1; kvinne; finale</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2574,7 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>5. kvinne; finale</t>
+          <t>5; kvinne; finale</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2626,7 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne; finale</t>
+          <t>7; kvinne; finale</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2678,7 @@
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>8. kvinne; finale; PB</t>
+          <t>8; kvinne; finale; PB</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2730,7 @@
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne; finsk mester; relatert utøver; Jyväskylä, Finland</t>
+          <t>1; kvinne; finsk mester; Jyväskylä, Finland</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>8. mann; totalplass 8; M25-29 klasse 1; SK Vidar-relatert; klubb i resultat Rørleggerkilebil</t>
+          <t>8; mann; totalplass 8; M25-29 klasse 1; klubb i resultat Rørleggerkilebil</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>9. mann; totalplass 9; M25-29 klasse 2; SK Vidar-relatert; klubb i resultat Oslo; nasjon i resultat USA</t>
+          <t>9; mann; totalplass 9; M25-29 klasse 2; klubb i resultat Oslo; nasjon i resultat USA</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2886,7 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>10. mann; totalplass 10; M30-34 klasse 3</t>
+          <t>10; mann; totalplass 10; M30-34 klasse 3</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne; totalplass 23; K25-29 klasse 1</t>
+          <t>2; kvinne; totalplass 23; K25-29 klasse 1</t>
         </is>
       </c>
     </row>
@@ -2990,7 +2990,7 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>5. kvinne; finale</t>
+          <t>5; kvinne; finale</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne; para; finale</t>
+          <t>1; kvinne; para; finale</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3142,7 @@
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne; finale</t>
+          <t>2; kvinne; finale</t>
         </is>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>13. mann; finale; Heat 2</t>
+          <t>13; mann; finale; Heat 2</t>
         </is>
       </c>
     </row>
@@ -3294,7 +3294,7 @@
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>22. mann; finale; Heat 1; PB</t>
+          <t>22; mann; finale; Heat 1; PB</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>36. mann; finale; Heat 1</t>
+          <t>36; mann; finale; Heat 1</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>39. mann; finale; Heat 1</t>
+          <t>39; mann; finale; Heat 1</t>
         </is>
       </c>
     </row>
@@ -3450,7 +3450,7 @@
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne; finale; Heat 2; SB</t>
+          <t>1; kvinne; finale; Heat 2; SB</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne; finale; Heat 2</t>
+          <t>2; kvinne; finale; Heat 2</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>4. kvinne; finale; Heat 2; SB</t>
+          <t>4; kvinne; finale; Heat 2; SB</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne; finale; Heat 2</t>
+          <t>7; kvinne; finale; Heat 2</t>
         </is>
       </c>
     </row>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>10. kvinne; finale; Heat 2</t>
+          <t>10; kvinne; finale; Heat 2</t>
         </is>
       </c>
     </row>
@@ -3710,7 +3710,7 @@
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>13. kvinne; finale; Heat 1; PB</t>
+          <t>13; kvinne; finale; Heat 1; PB</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3762,7 @@
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>16. kvinne; finale; Heat 1</t>
+          <t>16; kvinne; finale; Heat 1</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>17. kvinne; finale; Heat 1</t>
+          <t>17; kvinne; finale; Heat 1</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>8. kvinne; klasse 2; totalplass 41; registrert passering 23 min 02.9 sek; fra passering til mål 17 min 09.9 sek</t>
+          <t>8; kvinne; klasse 2; totalplass 41; registrert passering 23 min 02.9 sek; fra passering til mål 17 min 09.9 sek</t>
         </is>
       </c>
     </row>
@@ -4018,7 +4018,7 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>relatert utøver; Gjøvik Friidrettsklubb; ikke offisiell SK Vidar</t>
+          <t>Gjøvik Friidrettsklubb; ikke offisiell SK Vidar</t>
         </is>
       </c>
     </row>
@@ -4174,7 +4174,7 @@
       </c>
       <c r="J77" s="7" t="inlineStr">
         <is>
-          <t>1. plass</t>
+          <t>1; plass</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="J78" s="7" t="inlineStr">
         <is>
-          <t>2. mann, klasse 1</t>
+          <t>2; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J82" s="7" t="inlineStr">
         <is>
-          <t>6. kvinne, klasse 6</t>
+          <t>6; kvinne, klasse 6</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J83" s="7" t="inlineStr">
         <is>
-          <t>29. mann, klasse 29</t>
+          <t>29; mann, klasse 29</t>
         </is>
       </c>
     </row>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="J84" s="7" t="inlineStr">
         <is>
-          <t>6. kvinne, klasse 6</t>
+          <t>6; kvinne, klasse 6</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="J87" s="7" t="inlineStr">
         <is>
-          <t>1. totalt, klasse 1, ca. 1620 hm</t>
+          <t>1; totalt, klasse 1, ca; 1620 hm</t>
         </is>
       </c>
     </row>
@@ -4734,7 +4734,7 @@
       </c>
       <c r="J88" s="7" t="inlineStr">
         <is>
-          <t>8. totalt, klasse 3, ca. 1620 hm</t>
+          <t>8; totalt, klasse 3, ca; 1620 hm</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="J89" s="7" t="inlineStr">
         <is>
-          <t>klasse 1, 9. kvinne</t>
+          <t>klasse 1, 9; kvinne</t>
         </is>
       </c>
     </row>
@@ -4838,7 +4838,7 @@
       </c>
       <c r="J90" s="7" t="inlineStr">
         <is>
-          <t>klasse 7, 33. mann</t>
+          <t>klasse 7, 33; mann</t>
         </is>
       </c>
     </row>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="J91" s="7" t="inlineStr">
         <is>
-          <t>klasse 1, 2. mann</t>
+          <t>klasse 1, 2; mann</t>
         </is>
       </c>
     </row>
@@ -4942,7 +4942,7 @@
       </c>
       <c r="J92" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne</t>
+          <t>3; kvinne</t>
         </is>
       </c>
     </row>
@@ -4994,7 +4994,7 @@
       </c>
       <c r="J93" s="7" t="inlineStr">
         <is>
-          <t>4. mann</t>
+          <t>4; mann</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5042,7 @@
       </c>
       <c r="J94" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="J95" s="7" t="inlineStr">
         <is>
-          <t>13. mann</t>
+          <t>13; mann</t>
         </is>
       </c>
     </row>
@@ -5138,7 +5138,7 @@
       </c>
       <c r="J96" s="7" t="inlineStr">
         <is>
-          <t>31. mann</t>
+          <t>31; mann</t>
         </is>
       </c>
     </row>
@@ -5186,7 +5186,7 @@
       </c>
       <c r="J97" s="7" t="inlineStr">
         <is>
-          <t>44. mann</t>
+          <t>44; mann</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="J98" s="7" t="inlineStr">
         <is>
-          <t>18. kvinne</t>
+          <t>18; kvinne</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5286,7 @@
       </c>
       <c r="J99" s="7" t="inlineStr">
         <is>
-          <t>4. kvinne, motbakke, 1030 moh</t>
+          <t>4; kvinne, motbakke, 1030 moh</t>
         </is>
       </c>
     </row>
@@ -5490,7 +5490,7 @@
       </c>
       <c r="J103" s="7" t="inlineStr">
         <is>
-          <t>EXP 32 km / 2100 hm; 139. kvinner; brukeroppgitt resultat; UTMB Live</t>
+          <t>EXP 32 km / 2100 hm; 139; kvinner; brukeroppgitt resultat; UTMB Live</t>
         </is>
       </c>
     </row>
@@ -5542,7 +5542,7 @@
       </c>
       <c r="J104" s="7" t="inlineStr">
         <is>
-          <t>Zermatt/St. Niklaus, Sveits; kilde Datasport</t>
+          <t>Zermatt/St; Niklaus, Sveits; kilde Datasport</t>
         </is>
       </c>
     </row>
@@ -5594,7 +5594,7 @@
       </c>
       <c r="J105" s="7" t="inlineStr">
         <is>
-          <t>Zermatt/St. Niklaus, Sveits; kilde Datasport</t>
+          <t>Zermatt/St; Niklaus, Sveits; kilde Datasport</t>
         </is>
       </c>
     </row>
@@ -6138,7 +6138,7 @@
       </c>
       <c r="J116" s="7" t="inlineStr">
         <is>
-          <t>SKY MASTER 18 km / 900 hm; 33. kvinner; brukeroppgitt resultat; UTMB Live</t>
+          <t>SKY MASTER 18 km / 900 hm; 33; kvinner; brukeroppgitt resultat; UTMB Live</t>
         </is>
       </c>
     </row>
@@ -7004,11 +7004,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="J134" s="7" t="inlineStr">
-        <is>
-          <t>Manuell oppdatering fra bruker; SK Vidar-relatert</t>
-        </is>
-      </c>
+      <c r="J134" s="7" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
@@ -7394,7 +7390,7 @@
       </c>
       <c r="J142" s="7" t="inlineStr">
         <is>
-          <t>PDA 55 km / 3300 hm; 117. menn; brukeroppgitt resultat; UTMB Live</t>
+          <t>PDA 55 km / 3300 hm; 117; menn; brukeroppgitt resultat; UTMB Live</t>
         </is>
       </c>
     </row>
@@ -7446,7 +7442,7 @@
       </c>
       <c r="J143" s="7" t="inlineStr">
         <is>
-          <t>1. mann, klasse 1</t>
+          <t>1; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -7542,7 +7538,7 @@
       </c>
       <c r="J145" s="7" t="inlineStr">
         <is>
-          <t>9. mann, klasse 3</t>
+          <t>9; mann, klasse 3</t>
         </is>
       </c>
     </row>
@@ -7594,7 +7590,7 @@
       </c>
       <c r="J146" s="7" t="inlineStr">
         <is>
-          <t>4. kvinne, klasse 4</t>
+          <t>4; kvinne, klasse 4</t>
         </is>
       </c>
     </row>
@@ -7646,7 +7642,7 @@
       </c>
       <c r="J147" s="7" t="inlineStr">
         <is>
-          <t>1. mann, klasse 1</t>
+          <t>1; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -7698,7 +7694,7 @@
       </c>
       <c r="J148" s="7" t="inlineStr">
         <is>
-          <t>42km du Mont-Blanc 42 km / 2540 hm; 2. kvinne; klasse 2; LiveTrail; UTMB/LiveTrail screenshot; Ida Amelie/Amalie alias kontrollert</t>
+          <t>42km du Mont-Blanc 42 km / 2540 hm; 2; kvinne; klasse 2; LiveTrail</t>
         </is>
       </c>
     </row>
@@ -7894,7 +7890,7 @@
       </c>
       <c r="J152" s="7" t="inlineStr">
         <is>
-          <t>5. mann, klasse 5</t>
+          <t>5; mann, klasse 5</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7942,7 @@
       </c>
       <c r="J153" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1; rettet fra Havmaraton til Halvmaraton</t>
+          <t>1; kvinne, klasse 1; rettet fra Havmaraton til Halvmaraton</t>
         </is>
       </c>
     </row>
@@ -7998,7 +7994,7 @@
       </c>
       <c r="J154" s="7" t="inlineStr">
         <is>
-          <t>23km du Mont-Blanc 23 km / 1680 hm; 28. kvinner; klasse 19; LiveTrail; sterk SK Vidar-kandidat</t>
+          <t>23km du Mont-Blanc 23 km / 1680 hm; 28; kvinner; klasse 19; LiveTrail; sterk SK Vidar-kandidat</t>
         </is>
       </c>
     </row>
@@ -8050,7 +8046,7 @@
       </c>
       <c r="J155" s="7" t="inlineStr">
         <is>
-          <t>23km du Mont-Blanc 23 km / 1680 hm; 64. kvinner; klasse 40; LiveTrail; mulig SK Vidar via Slack og Nye lopere</t>
+          <t>23km du Mont-Blanc 23 km / 1680 hm; 64; kvinner; klasse 40; LiveTrail</t>
         </is>
       </c>
     </row>
@@ -8102,7 +8098,7 @@
       </c>
       <c r="J156" s="7" t="inlineStr">
         <is>
-          <t>23km du Mont-Blanc 23 km / 1680 hm; 442. menn; klasse 14; LiveTrail; klubb SK Vidar / Team Kondis</t>
+          <t>23km du Mont-Blanc 23 km / 1680 hm; 442; menn; klasse 14; LiveTrail; klubb SK Vidar / Team Kondis</t>
         </is>
       </c>
     </row>
@@ -9874,7 +9870,7 @@
       </c>
       <c r="J192" s="7" t="inlineStr">
         <is>
-          <t>1. mann, CP1 1 36, CP2 2 47, CP3 4 25, min/km 5, 07</t>
+          <t>1; mann, CP1 1 36, CP2 2 47, CP3 4 25, min/km 5, 07</t>
         </is>
       </c>
     </row>
@@ -9978,7 +9974,7 @@
       </c>
       <c r="J194" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1, relatert treff</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -10030,7 +10026,7 @@
       </c>
       <c r="J195" s="7" t="inlineStr">
         <is>
-          <t>4. kvinne, klasse 3, relatert treff</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -10082,7 +10078,7 @@
       </c>
       <c r="J196" s="7" t="inlineStr">
         <is>
-          <t>1. mann, klasse 1</t>
+          <t>1; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -10134,7 +10130,7 @@
       </c>
       <c r="J197" s="7" t="inlineStr">
         <is>
-          <t>5. kvinne, klasse 5</t>
+          <t>5; kvinne, klasse 5</t>
         </is>
       </c>
     </row>
@@ -10186,7 +10182,7 @@
       </c>
       <c r="J198" s="7" t="inlineStr">
         <is>
-          <t>6. kvinne, klasse 6</t>
+          <t>6; kvinne, klasse 6</t>
         </is>
       </c>
     </row>
@@ -10238,7 +10234,7 @@
       </c>
       <c r="J199" s="7" t="inlineStr">
         <is>
-          <t>5. kvinne, klasse 1</t>
+          <t>5; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -10290,7 +10286,7 @@
       </c>
       <c r="J200" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 2</t>
+          <t>2; kvinne, klasse 2</t>
         </is>
       </c>
     </row>
@@ -10340,11 +10336,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="J201" s="7" t="inlineStr">
-        <is>
-          <t>relatert utøver, FIN</t>
-        </is>
-      </c>
+      <c r="J201" s="7" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
@@ -10550,7 +10542,7 @@
       </c>
       <c r="J205" s="7" t="inlineStr">
         <is>
-          <t>89. mann, klasse 84, relatert treff</t>
+          <t>89</t>
         </is>
       </c>
     </row>
@@ -10602,7 +10594,7 @@
       </c>
       <c r="J206" s="7" t="inlineStr">
         <is>
-          <t>17. mann, klasse 1</t>
+          <t>17; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -10654,7 +10646,7 @@
       </c>
       <c r="J207" s="7" t="inlineStr">
         <is>
-          <t>12. kvinne, klasse 1</t>
+          <t>12; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -10706,7 +10698,7 @@
       </c>
       <c r="J208" s="7" t="inlineStr">
         <is>
-          <t>10. mann, klasse 10, relatert treff</t>
+          <t>10</t>
         </is>
       </c>
     </row>
@@ -10758,7 +10750,7 @@
       </c>
       <c r="J209" s="7" t="inlineStr">
         <is>
-          <t>3. mann, klasse 3, relatert treff</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -10810,7 +10802,7 @@
       </c>
       <c r="J210" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1, relatert treff</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -10862,7 +10854,7 @@
       </c>
       <c r="J211" s="7" t="inlineStr">
         <is>
-          <t>23. mann, klasse 4</t>
+          <t>23; mann, klasse 4</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10906,7 @@
       </c>
       <c r="J212" s="7" t="inlineStr">
         <is>
-          <t>29. mann, klasse 1</t>
+          <t>29; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -10966,7 +10958,7 @@
       </c>
       <c r="J213" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1</t>
+          <t>1; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -11018,7 +11010,7 @@
       </c>
       <c r="J214" s="7" t="inlineStr">
         <is>
-          <t>11. mann, klasse 3</t>
+          <t>11; mann, klasse 3</t>
         </is>
       </c>
     </row>
@@ -11070,7 +11062,7 @@
       </c>
       <c r="J215" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 1</t>
+          <t>2; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -11122,7 +11114,7 @@
       </c>
       <c r="J216" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1</t>
+          <t>1; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -11174,7 +11166,7 @@
       </c>
       <c r="J217" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 2</t>
+          <t>2; kvinne, klasse 2</t>
         </is>
       </c>
     </row>
@@ -11226,7 +11218,7 @@
       </c>
       <c r="J218" s="7" t="inlineStr">
         <is>
-          <t>4. mann, klasse 1, relatert treff</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -11278,7 +11270,7 @@
       </c>
       <c r="J219" s="7" t="inlineStr">
         <is>
-          <t>1. mann, klasse 1</t>
+          <t>1; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -11330,7 +11322,7 @@
       </c>
       <c r="J220" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 1, relatert treff</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -11382,7 +11374,7 @@
       </c>
       <c r="J221" s="7" t="inlineStr">
         <is>
-          <t>117. mann, klasse 4</t>
+          <t>117; mann, klasse 4</t>
         </is>
       </c>
     </row>
@@ -11434,7 +11426,7 @@
       </c>
       <c r="J222" s="7" t="inlineStr">
         <is>
-          <t>52. kvinne, klasse 5</t>
+          <t>52; kvinne, klasse 5</t>
         </is>
       </c>
     </row>
@@ -11486,7 +11478,7 @@
       </c>
       <c r="J223" s="7" t="inlineStr">
         <is>
-          <t>36. kvinne, klasse 15, relatert treff</t>
+          <t>36</t>
         </is>
       </c>
     </row>
@@ -11538,7 +11530,7 @@
       </c>
       <c r="J224" s="7" t="inlineStr">
         <is>
-          <t>3. mann, klasse 2</t>
+          <t>3; mann, klasse 2</t>
         </is>
       </c>
     </row>
@@ -11590,7 +11582,7 @@
       </c>
       <c r="J225" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1</t>
+          <t>1; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -11746,7 +11738,7 @@
       </c>
       <c r="J228" s="7" t="inlineStr">
         <is>
-          <t>597. mann, klasse 283</t>
+          <t>597; mann, klasse 283</t>
         </is>
       </c>
     </row>
@@ -11798,7 +11790,7 @@
       </c>
       <c r="J229" s="7" t="inlineStr">
         <is>
-          <t>3. mann, klasse 1</t>
+          <t>3; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -11850,7 +11842,7 @@
       </c>
       <c r="J230" s="7" t="inlineStr">
         <is>
-          <t>5. mann, klasse 1</t>
+          <t>5; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -11902,7 +11894,7 @@
       </c>
       <c r="J231" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 2</t>
+          <t>2; kvinne, klasse 2</t>
         </is>
       </c>
     </row>
@@ -11954,7 +11946,7 @@
       </c>
       <c r="J232" s="7" t="inlineStr">
         <is>
-          <t>30. mann, klasse 17</t>
+          <t>30; mann, klasse 17</t>
         </is>
       </c>
     </row>
@@ -12006,7 +11998,7 @@
       </c>
       <c r="J233" s="7" t="inlineStr">
         <is>
-          <t>19. mann, klasse 8</t>
+          <t>19; mann, klasse 8</t>
         </is>
       </c>
     </row>
@@ -12058,7 +12050,7 @@
       </c>
       <c r="J234" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1</t>
+          <t>1; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -12110,7 +12102,7 @@
       </c>
       <c r="J235" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 1</t>
+          <t>2; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -12162,7 +12154,7 @@
       </c>
       <c r="J236" s="7" t="inlineStr">
         <is>
-          <t>23. mann, klasse 10</t>
+          <t>23; mann, klasse 10</t>
         </is>
       </c>
     </row>
@@ -12214,7 +12206,7 @@
       </c>
       <c r="J237" s="7" t="inlineStr">
         <is>
-          <t>42. mann, klasse 8</t>
+          <t>42; mann, klasse 8</t>
         </is>
       </c>
     </row>
@@ -12266,7 +12258,7 @@
       </c>
       <c r="J238" s="7" t="inlineStr">
         <is>
-          <t>43. mann, klasse 20</t>
+          <t>43; mann, klasse 20</t>
         </is>
       </c>
     </row>
@@ -12318,7 +12310,7 @@
       </c>
       <c r="J239" s="7" t="inlineStr">
         <is>
-          <t>54. mann, klasse 4</t>
+          <t>54; mann, klasse 4</t>
         </is>
       </c>
     </row>
@@ -12370,7 +12362,7 @@
       </c>
       <c r="J240" s="7" t="inlineStr">
         <is>
-          <t>17. kvinne, klasse 1</t>
+          <t>17; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -12422,7 +12414,7 @@
       </c>
       <c r="J241" s="7" t="inlineStr">
         <is>
-          <t>18. kvinne, klasse 1</t>
+          <t>18; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -12474,7 +12466,7 @@
       </c>
       <c r="J242" s="7" t="inlineStr">
         <is>
-          <t>31. kvinne, klasse 15</t>
+          <t>31; kvinne, klasse 15</t>
         </is>
       </c>
     </row>
@@ -12526,7 +12518,7 @@
       </c>
       <c r="J243" s="7" t="inlineStr">
         <is>
-          <t>33. kvinne, klasse 16, relatert treff</t>
+          <t>33</t>
         </is>
       </c>
     </row>
@@ -12578,7 +12570,7 @@
       </c>
       <c r="J244" s="7" t="inlineStr">
         <is>
-          <t>140. mann, klasse 45</t>
+          <t>140; mann, klasse 45</t>
         </is>
       </c>
     </row>
@@ -12630,7 +12622,7 @@
       </c>
       <c r="J245" s="7" t="inlineStr">
         <is>
-          <t>238. mann, klasse 74</t>
+          <t>238; mann, klasse 74</t>
         </is>
       </c>
     </row>
@@ -12682,7 +12674,7 @@
       </c>
       <c r="J246" s="7" t="inlineStr">
         <is>
-          <t>97. kvinne, klasse 1</t>
+          <t>97; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -12734,7 +12726,7 @@
       </c>
       <c r="J247" s="7" t="inlineStr">
         <is>
-          <t>258. kvinne, klasse 28</t>
+          <t>258; kvinne, klasse 28</t>
         </is>
       </c>
     </row>
@@ -12786,7 +12778,7 @@
       </c>
       <c r="J248" s="7" t="inlineStr">
         <is>
-          <t>3. mann, klasse 2</t>
+          <t>3; mann, klasse 2</t>
         </is>
       </c>
     </row>
@@ -12838,7 +12830,7 @@
       </c>
       <c r="J249" s="7" t="inlineStr">
         <is>
-          <t>5. mann, klasse 3</t>
+          <t>5; mann, klasse 3</t>
         </is>
       </c>
     </row>
@@ -12890,7 +12882,7 @@
       </c>
       <c r="J250" s="7" t="inlineStr">
         <is>
-          <t>7. mann, klasse 4, relatert treff</t>
+          <t>7</t>
         </is>
       </c>
     </row>
@@ -12942,7 +12934,7 @@
       </c>
       <c r="J251" s="7" t="inlineStr">
         <is>
-          <t>11. kvinne, klasse 4, relatert treff</t>
+          <t>11</t>
         </is>
       </c>
     </row>
@@ -12994,7 +12986,7 @@
       </c>
       <c r="J252" s="7" t="inlineStr">
         <is>
-          <t>134. mann, klasse 17</t>
+          <t>134; mann, klasse 17</t>
         </is>
       </c>
     </row>
@@ -13046,7 +13038,7 @@
       </c>
       <c r="J253" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne, klasse 1</t>
+          <t>7; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -13098,7 +13090,7 @@
       </c>
       <c r="J254" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 1</t>
+          <t>2; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -13150,7 +13142,7 @@
       </c>
       <c r="J255" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne, klasse 3</t>
+          <t>7; kvinne, klasse 3</t>
         </is>
       </c>
     </row>
@@ -13200,11 +13192,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="J256" s="7" t="inlineStr">
-        <is>
-          <t>klasse 1, relatert treff</t>
-        </is>
-      </c>
+      <c r="J256" s="7" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" s="6" t="inlineStr">
@@ -13356,11 +13344,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="J259" s="7" t="inlineStr">
-        <is>
-          <t>klasse 1, relatert treff</t>
-        </is>
-      </c>
+      <c r="J259" s="7" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
@@ -13618,7 +13602,7 @@
       </c>
       <c r="J264" s="7" t="inlineStr">
         <is>
-          <t>145. kvinne, klasse 107</t>
+          <t>145; kvinne, klasse 107</t>
         </is>
       </c>
     </row>
@@ -13670,7 +13654,7 @@
       </c>
       <c r="J265" s="7" t="inlineStr">
         <is>
-          <t>154. kvinne, klasse 115</t>
+          <t>154; kvinne, klasse 115</t>
         </is>
       </c>
     </row>
@@ -13722,7 +13706,7 @@
       </c>
       <c r="J266" s="7" t="inlineStr">
         <is>
-          <t>164. kvinne, klasse 125</t>
+          <t>164; kvinne, klasse 125</t>
         </is>
       </c>
     </row>
@@ -13774,7 +13758,7 @@
       </c>
       <c r="J267" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne, klasse 4</t>
+          <t>7; kvinne, klasse 4</t>
         </is>
       </c>
     </row>
@@ -14704,11 +14688,7 @@
           <t>102</t>
         </is>
       </c>
-      <c r="J286" s="7" t="inlineStr">
-        <is>
-          <t>relatert treff</t>
-        </is>
-      </c>
+      <c r="J286" s="7" t="inlineStr"/>
     </row>
     <row r="287">
       <c r="A287" s="6" t="inlineStr">
@@ -14962,7 +14942,7 @@
       </c>
       <c r="J291" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 2</t>
+          <t>2; kvinne, klasse 2</t>
         </is>
       </c>
     </row>
@@ -15014,7 +14994,7 @@
       </c>
       <c r="J292" s="7" t="inlineStr">
         <is>
-          <t>3. mann, klasse 2, relatert treff</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -15066,7 +15046,7 @@
       </c>
       <c r="J293" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 1</t>
+          <t>2; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -15118,7 +15098,7 @@
       </c>
       <c r="J294" s="7" t="inlineStr">
         <is>
-          <t>35. mann, klasse 9, relatert treff</t>
+          <t>35</t>
         </is>
       </c>
     </row>
@@ -15222,7 +15202,7 @@
       </c>
       <c r="J296" s="7" t="inlineStr">
         <is>
-          <t>29. mann, klasse 11, relatert treff</t>
+          <t>29</t>
         </is>
       </c>
     </row>
@@ -15378,7 +15358,7 @@
       </c>
       <c r="J299" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -15430,7 +15410,7 @@
       </c>
       <c r="J300" s="7" t="inlineStr">
         <is>
-          <t>Pl. 1</t>
+          <t>Pl; 1</t>
         </is>
       </c>
     </row>
@@ -15638,7 +15618,7 @@
       </c>
       <c r="J304" s="7" t="inlineStr">
         <is>
-          <t>Pl. 4</t>
+          <t>Pl; 4</t>
         </is>
       </c>
     </row>
@@ -15738,7 +15718,7 @@
       </c>
       <c r="J306" s="7" t="inlineStr">
         <is>
-          <t>10. kvinne, klasse 2</t>
+          <t>10; kvinne, klasse 2</t>
         </is>
       </c>
     </row>
@@ -15790,7 +15770,7 @@
       </c>
       <c r="J307" s="7" t="inlineStr">
         <is>
-          <t>11. kvinne, klasse 7</t>
+          <t>11; kvinne, klasse 7</t>
         </is>
       </c>
     </row>
@@ -15842,7 +15822,7 @@
       </c>
       <c r="J308" s="7" t="inlineStr">
         <is>
-          <t>13. kvinne, klasse 3</t>
+          <t>13; kvinne, klasse 3</t>
         </is>
       </c>
     </row>
@@ -16134,7 +16114,7 @@
       </c>
       <c r="J314" s="7" t="inlineStr">
         <is>
-          <t>45. kvinne, klasse 6</t>
+          <t>45; kvinne, klasse 6</t>
         </is>
       </c>
     </row>
@@ -16186,7 +16166,7 @@
       </c>
       <c r="J315" s="7" t="inlineStr">
         <is>
-          <t>58. kvinne, klasse 14</t>
+          <t>58; kvinne, klasse 14</t>
         </is>
       </c>
     </row>
@@ -16286,7 +16266,7 @@
       </c>
       <c r="J317" s="7" t="inlineStr">
         <is>
-          <t>64. kvinne, klasse 6</t>
+          <t>64; kvinne, klasse 6</t>
         </is>
       </c>
     </row>
@@ -16338,7 +16318,7 @@
       </c>
       <c r="J318" s="7" t="inlineStr">
         <is>
-          <t>100. kvinne, klasse 5</t>
+          <t>100; kvinne, klasse 5</t>
         </is>
       </c>
     </row>
@@ -16390,7 +16370,7 @@
       </c>
       <c r="J319" s="7" t="inlineStr">
         <is>
-          <t>16. kvinne</t>
+          <t>16; kvinne</t>
         </is>
       </c>
     </row>
@@ -16442,7 +16422,7 @@
       </c>
       <c r="J320" s="7" t="inlineStr">
         <is>
-          <t>20. kvinne</t>
+          <t>20; kvinne</t>
         </is>
       </c>
     </row>
@@ -16494,7 +16474,7 @@
       </c>
       <c r="J321" s="7" t="inlineStr">
         <is>
-          <t>23. kvinne</t>
+          <t>23; kvinne</t>
         </is>
       </c>
     </row>
@@ -16546,7 +16526,7 @@
       </c>
       <c r="J322" s="7" t="inlineStr">
         <is>
-          <t>30. kvinne</t>
+          <t>30; kvinne</t>
         </is>
       </c>
     </row>
@@ -16598,7 +16578,7 @@
       </c>
       <c r="J323" s="7" t="inlineStr">
         <is>
-          <t>67. kvinne</t>
+          <t>67; kvinne</t>
         </is>
       </c>
     </row>
@@ -16650,7 +16630,7 @@
       </c>
       <c r="J324" s="7" t="inlineStr">
         <is>
-          <t>Pl. 7</t>
+          <t>Pl; 7</t>
         </is>
       </c>
     </row>
@@ -16702,7 +16682,7 @@
       </c>
       <c r="J325" s="7" t="inlineStr">
         <is>
-          <t>13. kvinne, klasse 7</t>
+          <t>13; kvinne, klasse 7</t>
         </is>
       </c>
     </row>
@@ -16754,7 +16734,7 @@
       </c>
       <c r="J326" s="7" t="inlineStr">
         <is>
-          <t>18. kvinne, klasse 5</t>
+          <t>18; kvinne, klasse 5</t>
         </is>
       </c>
     </row>
@@ -16806,7 +16786,7 @@
       </c>
       <c r="J327" s="7" t="inlineStr">
         <is>
-          <t>99. kvinne, klasse 1</t>
+          <t>99; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -16858,7 +16838,7 @@
       </c>
       <c r="J328" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -16910,7 +16890,7 @@
       </c>
       <c r="J329" s="7" t="inlineStr">
         <is>
-          <t>8. kvinne</t>
+          <t>8; kvinne</t>
         </is>
       </c>
     </row>
@@ -16962,7 +16942,7 @@
       </c>
       <c r="J330" s="7" t="inlineStr">
         <is>
-          <t>13. kvinne</t>
+          <t>13; kvinne</t>
         </is>
       </c>
     </row>
@@ -17014,7 +16994,7 @@
       </c>
       <c r="J331" s="7" t="inlineStr">
         <is>
-          <t>21. kvinne</t>
+          <t>21; kvinne</t>
         </is>
       </c>
     </row>
@@ -17066,7 +17046,7 @@
       </c>
       <c r="J332" s="7" t="inlineStr">
         <is>
-          <t>5. mann</t>
+          <t>5; mann</t>
         </is>
       </c>
     </row>
@@ -17118,7 +17098,7 @@
       </c>
       <c r="J333" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne</t>
+          <t>3; kvinne</t>
         </is>
       </c>
     </row>
@@ -17170,7 +17150,7 @@
       </c>
       <c r="J334" s="7" t="inlineStr">
         <is>
-          <t>8. kvinne</t>
+          <t>8; kvinne</t>
         </is>
       </c>
     </row>
@@ -17222,7 +17202,7 @@
       </c>
       <c r="J335" s="7" t="inlineStr">
         <is>
-          <t>104. mann</t>
+          <t>104; mann</t>
         </is>
       </c>
     </row>
@@ -17274,7 +17254,7 @@
       </c>
       <c r="J336" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -17326,7 +17306,7 @@
       </c>
       <c r="J337" s="7" t="inlineStr">
         <is>
-          <t>2. mann, klasse 2</t>
+          <t>2; mann, klasse 2</t>
         </is>
       </c>
     </row>
@@ -17378,7 +17358,7 @@
       </c>
       <c r="J338" s="7" t="inlineStr">
         <is>
-          <t>4. mann, klasse 1</t>
+          <t>4; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -17430,7 +17410,7 @@
       </c>
       <c r="J339" s="7" t="inlineStr">
         <is>
-          <t>6. mann, klasse 4</t>
+          <t>6; mann, klasse 4</t>
         </is>
       </c>
     </row>
@@ -17482,7 +17462,7 @@
       </c>
       <c r="J340" s="7" t="inlineStr">
         <is>
-          <t>8. mann, klasse 6</t>
+          <t>8; mann, klasse 6</t>
         </is>
       </c>
     </row>
@@ -17534,7 +17514,7 @@
       </c>
       <c r="J341" s="7" t="inlineStr">
         <is>
-          <t>9. mann, klasse 7</t>
+          <t>9; mann, klasse 7</t>
         </is>
       </c>
     </row>
@@ -17586,7 +17566,7 @@
       </c>
       <c r="J342" s="7" t="inlineStr">
         <is>
-          <t>11. mann, klasse 9</t>
+          <t>11; mann, klasse 9</t>
         </is>
       </c>
     </row>
@@ -17638,7 +17618,7 @@
       </c>
       <c r="J343" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1</t>
+          <t>1; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -17690,7 +17670,7 @@
       </c>
       <c r="J344" s="7" t="inlineStr">
         <is>
-          <t>14. mann, klasse 2</t>
+          <t>14; mann, klasse 2</t>
         </is>
       </c>
     </row>
@@ -17742,7 +17722,7 @@
       </c>
       <c r="J345" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne, klasse 2</t>
+          <t>2; kvinne, klasse 2</t>
         </is>
       </c>
     </row>
@@ -17794,7 +17774,7 @@
       </c>
       <c r="J346" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne, klasse 3</t>
+          <t>3; kvinne, klasse 3</t>
         </is>
       </c>
     </row>
@@ -17846,7 +17826,7 @@
       </c>
       <c r="J347" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne, klasse 6</t>
+          <t>7; kvinne, klasse 6</t>
         </is>
       </c>
     </row>
@@ -17898,7 +17878,7 @@
       </c>
       <c r="J348" s="7" t="inlineStr">
         <is>
-          <t>46. mann, klasse 5</t>
+          <t>46; mann, klasse 5</t>
         </is>
       </c>
     </row>
@@ -17950,7 +17930,7 @@
       </c>
       <c r="J349" s="7" t="inlineStr">
         <is>
-          <t>8. kvinne, klasse 7</t>
+          <t>8; kvinne, klasse 7</t>
         </is>
       </c>
     </row>
@@ -18002,7 +17982,7 @@
       </c>
       <c r="J350" s="7" t="inlineStr">
         <is>
-          <t>9. kvinne, klasse 8</t>
+          <t>9; kvinne, klasse 8</t>
         </is>
       </c>
     </row>
@@ -18054,7 +18034,7 @@
       </c>
       <c r="J351" s="7" t="inlineStr">
         <is>
-          <t>62. mann, klasse 1</t>
+          <t>62; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -18106,7 +18086,7 @@
       </c>
       <c r="J352" s="7" t="inlineStr">
         <is>
-          <t>12. kvinne, klasse 1</t>
+          <t>12; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -18158,7 +18138,7 @@
       </c>
       <c r="J353" s="7" t="inlineStr">
         <is>
-          <t>13. kvinne, klasse 1</t>
+          <t>13; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -18210,7 +18190,7 @@
       </c>
       <c r="J354" s="7" t="inlineStr">
         <is>
-          <t>77. mann, klasse 15</t>
+          <t>77; mann, klasse 15</t>
         </is>
       </c>
     </row>
@@ -18262,7 +18242,7 @@
       </c>
       <c r="J355" s="7" t="inlineStr">
         <is>
-          <t>14. kvinne, klasse 1</t>
+          <t>14; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -18314,7 +18294,7 @@
       </c>
       <c r="J356" s="7" t="inlineStr">
         <is>
-          <t>82. mann, klasse 40</t>
+          <t>82; mann, klasse 40</t>
         </is>
       </c>
     </row>
@@ -18366,7 +18346,7 @@
       </c>
       <c r="J357" s="7" t="inlineStr">
         <is>
-          <t>15. kvinne, klasse 10</t>
+          <t>15; kvinne, klasse 10</t>
         </is>
       </c>
     </row>
@@ -18418,7 +18398,7 @@
       </c>
       <c r="J358" s="7" t="inlineStr">
         <is>
-          <t>114. mann, klasse 55</t>
+          <t>114; mann, klasse 55</t>
         </is>
       </c>
     </row>
@@ -18470,7 +18450,7 @@
       </c>
       <c r="J359" s="7" t="inlineStr">
         <is>
-          <t>34. kvinne, klasse 18</t>
+          <t>34; kvinne, klasse 18</t>
         </is>
       </c>
     </row>
@@ -18522,7 +18502,7 @@
       </c>
       <c r="J360" s="7" t="inlineStr">
         <is>
-          <t>38. kvinne, klasse 1</t>
+          <t>38; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -18574,7 +18554,7 @@
       </c>
       <c r="J361" s="7" t="inlineStr">
         <is>
-          <t>52. kvinne, klasse 6</t>
+          <t>52; kvinne, klasse 6</t>
         </is>
       </c>
     </row>
@@ -18626,7 +18606,7 @@
       </c>
       <c r="J362" s="7" t="inlineStr">
         <is>
-          <t>61. kvinne, klasse 5</t>
+          <t>61; kvinne, klasse 5</t>
         </is>
       </c>
     </row>
@@ -18678,7 +18658,7 @@
       </c>
       <c r="J363" s="7" t="inlineStr">
         <is>
-          <t>278. mann, klasse 2</t>
+          <t>278; mann, klasse 2</t>
         </is>
       </c>
     </row>
@@ -18730,7 +18710,7 @@
       </c>
       <c r="J364" s="7" t="inlineStr">
         <is>
-          <t>2. mann, klasse 2</t>
+          <t>2; mann, klasse 2</t>
         </is>
       </c>
     </row>
@@ -18782,7 +18762,7 @@
       </c>
       <c r="J365" s="7" t="inlineStr">
         <is>
-          <t>6. mann, klasse 1</t>
+          <t>6; mann, klasse 1</t>
         </is>
       </c>
     </row>
@@ -18834,7 +18814,7 @@
       </c>
       <c r="J366" s="7" t="inlineStr">
         <is>
-          <t>10. mann, klasse 7</t>
+          <t>10; mann, klasse 7</t>
         </is>
       </c>
     </row>
@@ -18886,7 +18866,7 @@
       </c>
       <c r="J367" s="7" t="inlineStr">
         <is>
-          <t>11. mann, klasse 8</t>
+          <t>11; mann, klasse 8</t>
         </is>
       </c>
     </row>
@@ -18938,7 +18918,7 @@
       </c>
       <c r="J368" s="7" t="inlineStr">
         <is>
-          <t>14. mann, klasse 11</t>
+          <t>14; mann, klasse 11</t>
         </is>
       </c>
     </row>
@@ -18990,7 +18970,7 @@
       </c>
       <c r="J369" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, klasse 1</t>
+          <t>1; kvinne, klasse 1</t>
         </is>
       </c>
     </row>
@@ -19042,7 +19022,7 @@
       </c>
       <c r="J370" s="7" t="inlineStr">
         <is>
-          <t>46. mann, klasse 26</t>
+          <t>46; mann, klasse 26</t>
         </is>
       </c>
     </row>
@@ -19094,7 +19074,7 @@
       </c>
       <c r="J371" s="7" t="inlineStr">
         <is>
-          <t>79. mann, klasse 37</t>
+          <t>79; mann, klasse 37</t>
         </is>
       </c>
     </row>
@@ -19146,7 +19126,7 @@
       </c>
       <c r="J372" s="7" t="inlineStr">
         <is>
-          <t>10. kvinne, klasse 8</t>
+          <t>10; kvinne, klasse 8</t>
         </is>
       </c>
     </row>
@@ -19198,7 +19178,7 @@
       </c>
       <c r="J373" s="7" t="inlineStr">
         <is>
-          <t>11. kvinne, klasse 9</t>
+          <t>11; kvinne, klasse 9</t>
         </is>
       </c>
     </row>
@@ -19250,7 +19230,7 @@
       </c>
       <c r="J374" s="7" t="inlineStr">
         <is>
-          <t>135. mann, klasse 3</t>
+          <t>135; mann, klasse 3</t>
         </is>
       </c>
     </row>
@@ -19302,7 +19282,7 @@
       </c>
       <c r="J375" s="7" t="inlineStr">
         <is>
-          <t>174. mann, klasse 24</t>
+          <t>174; mann, klasse 24</t>
         </is>
       </c>
     </row>
@@ -19354,7 +19334,7 @@
       </c>
       <c r="J376" s="7" t="inlineStr">
         <is>
-          <t>222. mann, klasse 85</t>
+          <t>222; mann, klasse 85</t>
         </is>
       </c>
     </row>
@@ -19406,7 +19386,7 @@
       </c>
       <c r="J377" s="7" t="inlineStr">
         <is>
-          <t>230. mann, klasse 50</t>
+          <t>230; mann, klasse 50</t>
         </is>
       </c>
     </row>
@@ -19458,7 +19438,7 @@
       </c>
       <c r="J378" s="7" t="inlineStr">
         <is>
-          <t>243. mann, klasse 11</t>
+          <t>243; mann, klasse 11</t>
         </is>
       </c>
     </row>
@@ -19510,7 +19490,7 @@
       </c>
       <c r="J379" s="7" t="inlineStr">
         <is>
-          <t>317. mann, klasse 43</t>
+          <t>317; mann, klasse 43</t>
         </is>
       </c>
     </row>
@@ -19562,7 +19542,7 @@
       </c>
       <c r="J380" s="7" t="inlineStr">
         <is>
-          <t>97. kvinne, klasse 12</t>
+          <t>97; kvinne, klasse 12</t>
         </is>
       </c>
     </row>
@@ -20726,7 +20706,7 @@
       </c>
       <c r="J404" s="7" t="inlineStr">
         <is>
-          <t>6. mann</t>
+          <t>6; mann</t>
         </is>
       </c>
     </row>
@@ -20778,7 +20758,7 @@
       </c>
       <c r="J405" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -20830,7 +20810,7 @@
       </c>
       <c r="J406" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne</t>
+          <t>3; kvinne</t>
         </is>
       </c>
     </row>
@@ -20882,7 +20862,7 @@
       </c>
       <c r="J407" s="7" t="inlineStr">
         <is>
-          <t>24. kvinne</t>
+          <t>24; kvinne</t>
         </is>
       </c>
     </row>
@@ -20934,7 +20914,7 @@
       </c>
       <c r="J408" s="7" t="inlineStr">
         <is>
-          <t>199. mann</t>
+          <t>199; mann</t>
         </is>
       </c>
     </row>
@@ -20986,7 +20966,7 @@
       </c>
       <c r="J409" s="7" t="inlineStr">
         <is>
-          <t>139. kvinne</t>
+          <t>139; kvinne</t>
         </is>
       </c>
     </row>
@@ -21038,7 +21018,7 @@
       </c>
       <c r="J410" s="7" t="inlineStr">
         <is>
-          <t>2. mann</t>
+          <t>2; mann</t>
         </is>
       </c>
     </row>
@@ -21090,7 +21070,7 @@
       </c>
       <c r="J411" s="7" t="inlineStr">
         <is>
-          <t>22. kvinne</t>
+          <t>22; kvinne</t>
         </is>
       </c>
     </row>
@@ -21142,7 +21122,7 @@
       </c>
       <c r="J412" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -21194,7 +21174,7 @@
       </c>
       <c r="J413" s="7" t="inlineStr">
         <is>
-          <t>77. mann</t>
+          <t>77; mann</t>
         </is>
       </c>
     </row>
@@ -21246,7 +21226,7 @@
       </c>
       <c r="J414" s="7" t="inlineStr">
         <is>
-          <t>2. mann</t>
+          <t>2; mann</t>
         </is>
       </c>
     </row>
@@ -21298,7 +21278,7 @@
       </c>
       <c r="J415" s="7" t="inlineStr">
         <is>
-          <t>5. kvinne</t>
+          <t>5; kvinne</t>
         </is>
       </c>
     </row>
@@ -21350,7 +21330,7 @@
       </c>
       <c r="J416" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -21402,7 +21382,7 @@
       </c>
       <c r="J417" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne</t>
+          <t>7; kvinne</t>
         </is>
       </c>
     </row>
@@ -21506,7 +21486,7 @@
       </c>
       <c r="J419" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -21610,7 +21590,7 @@
       </c>
       <c r="J421" s="7" t="inlineStr">
         <is>
-          <t>64. kvinne</t>
+          <t>64; kvinne</t>
         </is>
       </c>
     </row>
@@ -22058,7 +22038,7 @@
       </c>
       <c r="J431" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -22110,7 +22090,7 @@
       </c>
       <c r="J432" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -22162,7 +22142,7 @@
       </c>
       <c r="J433" s="7" t="inlineStr">
         <is>
-          <t>6. kvinne</t>
+          <t>6; kvinne</t>
         </is>
       </c>
     </row>
@@ -22214,7 +22194,7 @@
       </c>
       <c r="J434" s="7" t="inlineStr">
         <is>
-          <t>220. mann</t>
+          <t>220; mann</t>
         </is>
       </c>
     </row>
@@ -22266,7 +22246,7 @@
       </c>
       <c r="J435" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -22314,7 +22294,7 @@
       <c r="I436" s="7" t="inlineStr"/>
       <c r="J436" s="7" t="inlineStr">
         <is>
-          <t>5. kvinne</t>
+          <t>5; kvinne</t>
         </is>
       </c>
     </row>
@@ -22362,7 +22342,7 @@
       <c r="I437" s="7" t="inlineStr"/>
       <c r="J437" s="7" t="inlineStr">
         <is>
-          <t>7. kvinne</t>
+          <t>7; kvinne</t>
         </is>
       </c>
     </row>
@@ -23478,7 +23458,7 @@
       </c>
       <c r="J459" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -23530,7 +23510,7 @@
       </c>
       <c r="J460" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -23582,7 +23562,7 @@
       </c>
       <c r="J461" s="7" t="inlineStr">
         <is>
-          <t>9. kvinne</t>
+          <t>9; kvinne</t>
         </is>
       </c>
     </row>
@@ -23634,7 +23614,7 @@
       </c>
       <c r="J462" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -23738,7 +23718,7 @@
       </c>
       <c r="J464" s="7" t="inlineStr">
         <is>
-          <t>6. plass menn</t>
+          <t>6; plass menn</t>
         </is>
       </c>
     </row>
@@ -23790,7 +23770,7 @@
       </c>
       <c r="J465" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -23842,7 +23822,7 @@
       </c>
       <c r="J466" s="7" t="inlineStr">
         <is>
-          <t>8. mann</t>
+          <t>8; mann</t>
         </is>
       </c>
     </row>
@@ -23894,7 +23874,7 @@
       </c>
       <c r="J467" s="7" t="inlineStr">
         <is>
-          <t>16. mann</t>
+          <t>16; mann</t>
         </is>
       </c>
     </row>
@@ -23946,7 +23926,7 @@
       </c>
       <c r="J468" s="7" t="inlineStr">
         <is>
-          <t>27. mann</t>
+          <t>27; mann</t>
         </is>
       </c>
     </row>
@@ -23998,7 +23978,7 @@
       </c>
       <c r="J469" s="7" t="inlineStr">
         <is>
-          <t>30. mann</t>
+          <t>30; mann</t>
         </is>
       </c>
     </row>
@@ -24050,7 +24030,7 @@
       </c>
       <c r="J470" s="7" t="inlineStr">
         <is>
-          <t>66. mann</t>
+          <t>66; mann</t>
         </is>
       </c>
     </row>
@@ -24102,7 +24082,7 @@
       </c>
       <c r="J471" s="7" t="inlineStr">
         <is>
-          <t>67. mann</t>
+          <t>67; mann</t>
         </is>
       </c>
     </row>
@@ -24154,7 +24134,7 @@
       </c>
       <c r="J472" s="7" t="inlineStr">
         <is>
-          <t>109. mann</t>
+          <t>109; mann</t>
         </is>
       </c>
     </row>
@@ -24206,7 +24186,7 @@
       </c>
       <c r="J473" s="7" t="inlineStr">
         <is>
-          <t>113. mann</t>
+          <t>113; mann</t>
         </is>
       </c>
     </row>
@@ -24258,7 +24238,7 @@
       </c>
       <c r="J474" s="7" t="inlineStr">
         <is>
-          <t>16. kvinne</t>
+          <t>16; kvinne</t>
         </is>
       </c>
     </row>
@@ -24310,7 +24290,7 @@
       </c>
       <c r="J475" s="7" t="inlineStr">
         <is>
-          <t>33. kvinne</t>
+          <t>33; kvinne</t>
         </is>
       </c>
     </row>
@@ -24362,7 +24342,7 @@
       </c>
       <c r="J476" s="7" t="inlineStr">
         <is>
-          <t>215. mann</t>
+          <t>215; mann</t>
         </is>
       </c>
     </row>
@@ -24414,7 +24394,7 @@
       </c>
       <c r="J477" s="7" t="inlineStr">
         <is>
-          <t>54. kvinne</t>
+          <t>54; kvinne</t>
         </is>
       </c>
     </row>
@@ -24466,7 +24446,7 @@
       </c>
       <c r="J478" s="7" t="inlineStr">
         <is>
-          <t>247. mann</t>
+          <t>247; mann</t>
         </is>
       </c>
     </row>
@@ -24518,7 +24498,7 @@
       </c>
       <c r="J479" s="7" t="inlineStr">
         <is>
-          <t>254. mann</t>
+          <t>254; mann</t>
         </is>
       </c>
     </row>
@@ -24570,7 +24550,7 @@
       </c>
       <c r="J480" s="7" t="inlineStr">
         <is>
-          <t>182. kvinne</t>
+          <t>182; kvinne</t>
         </is>
       </c>
     </row>
@@ -24622,7 +24602,7 @@
       </c>
       <c r="J481" s="7" t="inlineStr">
         <is>
-          <t>10. plass menn</t>
+          <t>10; plass menn</t>
         </is>
       </c>
     </row>
@@ -25062,7 +25042,7 @@
       </c>
       <c r="J490" s="7" t="inlineStr">
         <is>
-          <t>8. mann</t>
+          <t>8; mann</t>
         </is>
       </c>
     </row>
@@ -25114,7 +25094,7 @@
       </c>
       <c r="J491" s="7" t="inlineStr">
         <is>
-          <t>3. mann</t>
+          <t>3; mann</t>
         </is>
       </c>
     </row>
@@ -25166,7 +25146,7 @@
       </c>
       <c r="J492" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -25218,7 +25198,7 @@
       </c>
       <c r="J493" s="7" t="inlineStr">
         <is>
-          <t>12. mann</t>
+          <t>12; mann</t>
         </is>
       </c>
     </row>
@@ -25270,7 +25250,7 @@
       </c>
       <c r="J494" s="7" t="inlineStr">
         <is>
-          <t>4. kvinne</t>
+          <t>4; kvinne</t>
         </is>
       </c>
     </row>
@@ -25322,7 +25302,7 @@
       </c>
       <c r="J495" s="7" t="inlineStr">
         <is>
-          <t>20. kvinne</t>
+          <t>20; kvinne</t>
         </is>
       </c>
     </row>
@@ -25374,7 +25354,7 @@
       </c>
       <c r="J496" s="7" t="inlineStr">
         <is>
-          <t>3. mann</t>
+          <t>3; mann</t>
         </is>
       </c>
     </row>
@@ -25426,7 +25406,7 @@
       </c>
       <c r="J497" s="7" t="inlineStr">
         <is>
-          <t>6. mann</t>
+          <t>6; mann</t>
         </is>
       </c>
     </row>
@@ -25478,7 +25458,7 @@
       </c>
       <c r="J498" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -25530,7 +25510,7 @@
       </c>
       <c r="J499" s="7" t="inlineStr">
         <is>
-          <t>31. mann</t>
+          <t>31; mann</t>
         </is>
       </c>
     </row>
@@ -25582,7 +25562,7 @@
       </c>
       <c r="J500" s="7" t="inlineStr">
         <is>
-          <t>46. mann</t>
+          <t>46; mann</t>
         </is>
       </c>
     </row>
@@ -25634,7 +25614,7 @@
       </c>
       <c r="J501" s="7" t="inlineStr">
         <is>
-          <t>14. kvinne</t>
+          <t>14; kvinne</t>
         </is>
       </c>
     </row>
@@ -25686,7 +25666,7 @@
       </c>
       <c r="J502" s="7" t="inlineStr">
         <is>
-          <t>39. kvinne</t>
+          <t>39; kvinne</t>
         </is>
       </c>
     </row>
@@ -25738,7 +25718,7 @@
       </c>
       <c r="J503" s="7" t="inlineStr">
         <is>
-          <t>10. mann</t>
+          <t>10; mann</t>
         </is>
       </c>
     </row>
@@ -25790,7 +25770,7 @@
       </c>
       <c r="J504" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -25842,7 +25822,7 @@
       </c>
       <c r="J505" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne</t>
+          <t>3; kvinne</t>
         </is>
       </c>
     </row>
@@ -25894,7 +25874,7 @@
       </c>
       <c r="J506" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -25946,7 +25926,7 @@
       </c>
       <c r="J507" s="7" t="inlineStr">
         <is>
-          <t>11. kvinne</t>
+          <t>11; kvinne</t>
         </is>
       </c>
     </row>
@@ -26050,7 +26030,7 @@
       </c>
       <c r="J509" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -26150,7 +26130,7 @@
       </c>
       <c r="J511" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne</t>
+          <t>3; kvinne</t>
         </is>
       </c>
     </row>
@@ -26202,7 +26182,7 @@
       </c>
       <c r="J512" s="7" t="inlineStr">
         <is>
-          <t>1. M65-69</t>
+          <t>1; M65-69</t>
         </is>
       </c>
     </row>
@@ -26254,7 +26234,7 @@
       </c>
       <c r="J513" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -26306,7 +26286,7 @@
       </c>
       <c r="J514" s="7" t="inlineStr">
         <is>
-          <t>73. mann</t>
+          <t>73; mann</t>
         </is>
       </c>
     </row>
@@ -26402,7 +26382,7 @@
       </c>
       <c r="J516" s="7" t="inlineStr">
         <is>
-          <t>9. mann; 5. Herre 30-39</t>
+          <t>9; mann; 5; Herre 30-39</t>
         </is>
       </c>
     </row>
@@ -26454,7 +26434,7 @@
       </c>
       <c r="J517" s="7" t="inlineStr">
         <is>
-          <t>16. mann; 9. Herre 30-39</t>
+          <t>16; mann; 9; Herre 30-39</t>
         </is>
       </c>
     </row>
@@ -26506,7 +26486,7 @@
       </c>
       <c r="J518" s="7" t="inlineStr">
         <is>
-          <t>86. mann; 47. Herre 30-39</t>
+          <t>86; mann; 47; Herre 30-39</t>
         </is>
       </c>
     </row>
@@ -26558,7 +26538,7 @@
       </c>
       <c r="J519" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -26610,7 +26590,7 @@
       </c>
       <c r="J520" s="7" t="inlineStr">
         <is>
-          <t>6. mann</t>
+          <t>6; mann</t>
         </is>
       </c>
     </row>
@@ -26950,7 +26930,7 @@
       </c>
       <c r="J527" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -27002,7 +26982,7 @@
       </c>
       <c r="J528" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -27054,7 +27034,7 @@
       </c>
       <c r="J529" s="7" t="inlineStr">
         <is>
-          <t>6. mann</t>
+          <t>6; mann</t>
         </is>
       </c>
     </row>
@@ -27106,7 +27086,7 @@
       </c>
       <c r="J530" s="7" t="inlineStr">
         <is>
-          <t>7. mann</t>
+          <t>7; mann</t>
         </is>
       </c>
     </row>
@@ -27158,7 +27138,7 @@
       </c>
       <c r="J531" s="7" t="inlineStr">
         <is>
-          <t>10. mann</t>
+          <t>10; mann</t>
         </is>
       </c>
     </row>
@@ -27210,7 +27190,7 @@
       </c>
       <c r="J532" s="7" t="inlineStr">
         <is>
-          <t>11. mann</t>
+          <t>11; mann</t>
         </is>
       </c>
     </row>
@@ -27262,7 +27242,7 @@
       </c>
       <c r="J533" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -27314,7 +27294,7 @@
       </c>
       <c r="J534" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -27366,7 +27346,7 @@
       </c>
       <c r="J535" s="7" t="inlineStr">
         <is>
-          <t>32. mann</t>
+          <t>32; mann</t>
         </is>
       </c>
     </row>
@@ -27418,7 +27398,7 @@
       </c>
       <c r="J536" s="7" t="inlineStr">
         <is>
-          <t>38. mann</t>
+          <t>38; mann</t>
         </is>
       </c>
     </row>
@@ -27470,7 +27450,7 @@
       </c>
       <c r="J537" s="7" t="inlineStr">
         <is>
-          <t>57. mann</t>
+          <t>57; mann</t>
         </is>
       </c>
     </row>
@@ -27522,7 +27502,7 @@
       </c>
       <c r="J538" s="7" t="inlineStr">
         <is>
-          <t>57. mann</t>
+          <t>57; mann</t>
         </is>
       </c>
     </row>
@@ -27574,7 +27554,7 @@
       </c>
       <c r="J539" s="7" t="inlineStr">
         <is>
-          <t>63. mann</t>
+          <t>63; mann</t>
         </is>
       </c>
     </row>
@@ -27626,7 +27606,7 @@
       </c>
       <c r="J540" s="7" t="inlineStr">
         <is>
-          <t>9. kvinne</t>
+          <t>9; kvinne</t>
         </is>
       </c>
     </row>
@@ -27678,7 +27658,7 @@
       </c>
       <c r="J541" s="7" t="inlineStr">
         <is>
-          <t>10. kvinne</t>
+          <t>10; kvinne</t>
         </is>
       </c>
     </row>
@@ -27730,7 +27710,7 @@
       </c>
       <c r="J542" s="7" t="inlineStr">
         <is>
-          <t>11. kvinne</t>
+          <t>11; kvinne</t>
         </is>
       </c>
     </row>
@@ -27782,7 +27762,7 @@
       </c>
       <c r="J543" s="7" t="inlineStr">
         <is>
-          <t>79. mann</t>
+          <t>79; mann</t>
         </is>
       </c>
     </row>
@@ -27834,7 +27814,7 @@
       </c>
       <c r="J544" s="7" t="inlineStr">
         <is>
-          <t>14. kvinne</t>
+          <t>14; kvinne</t>
         </is>
       </c>
     </row>
@@ -27886,7 +27866,7 @@
       </c>
       <c r="J545" s="7" t="inlineStr">
         <is>
-          <t>104. mann</t>
+          <t>104; mann</t>
         </is>
       </c>
     </row>
@@ -27938,7 +27918,7 @@
       </c>
       <c r="J546" s="7" t="inlineStr">
         <is>
-          <t>124. mann</t>
+          <t>124; mann</t>
         </is>
       </c>
     </row>
@@ -27990,7 +27970,7 @@
       </c>
       <c r="J547" s="7" t="inlineStr">
         <is>
-          <t>129. mann</t>
+          <t>129; mann</t>
         </is>
       </c>
     </row>
@@ -28042,7 +28022,7 @@
       </c>
       <c r="J548" s="7" t="inlineStr">
         <is>
-          <t>26. kvinne</t>
+          <t>26; kvinne</t>
         </is>
       </c>
     </row>
@@ -28094,7 +28074,7 @@
       </c>
       <c r="J549" s="7" t="inlineStr">
         <is>
-          <t>142. mann</t>
+          <t>142; mann</t>
         </is>
       </c>
     </row>
@@ -28146,7 +28126,7 @@
       </c>
       <c r="J550" s="7" t="inlineStr">
         <is>
-          <t>30. kvinne</t>
+          <t>30; kvinne</t>
         </is>
       </c>
     </row>
@@ -28198,7 +28178,7 @@
       </c>
       <c r="J551" s="7" t="inlineStr">
         <is>
-          <t>33. kvinne</t>
+          <t>33; kvinne</t>
         </is>
       </c>
     </row>
@@ -28250,7 +28230,7 @@
       </c>
       <c r="J552" s="7" t="inlineStr">
         <is>
-          <t>36. kvinne</t>
+          <t>36; kvinne</t>
         </is>
       </c>
     </row>
@@ -28302,7 +28282,7 @@
       </c>
       <c r="J553" s="7" t="inlineStr">
         <is>
-          <t>170. mann</t>
+          <t>170; mann</t>
         </is>
       </c>
     </row>
@@ -28354,7 +28334,7 @@
       </c>
       <c r="J554" s="7" t="inlineStr">
         <is>
-          <t>40. kvinne</t>
+          <t>40; kvinne</t>
         </is>
       </c>
     </row>
@@ -28406,7 +28386,7 @@
       </c>
       <c r="J555" s="7" t="inlineStr">
         <is>
-          <t>171. mann</t>
+          <t>171; mann</t>
         </is>
       </c>
     </row>
@@ -28458,7 +28438,7 @@
       </c>
       <c r="J556" s="7" t="inlineStr">
         <is>
-          <t>50. kvinne</t>
+          <t>50; kvinne</t>
         </is>
       </c>
     </row>
@@ -28510,7 +28490,7 @@
       </c>
       <c r="J557" s="7" t="inlineStr">
         <is>
-          <t>213. mann</t>
+          <t>213; mann</t>
         </is>
       </c>
     </row>
@@ -28562,7 +28542,7 @@
       </c>
       <c r="J558" s="7" t="inlineStr">
         <is>
-          <t>64. kvinne</t>
+          <t>64; kvinne</t>
         </is>
       </c>
     </row>
@@ -28614,7 +28594,7 @@
       </c>
       <c r="J559" s="7" t="inlineStr">
         <is>
-          <t>221. mann</t>
+          <t>221; mann</t>
         </is>
       </c>
     </row>
@@ -28666,7 +28646,7 @@
       </c>
       <c r="J560" s="7" t="inlineStr">
         <is>
-          <t>67. kvinne</t>
+          <t>67; kvinne</t>
         </is>
       </c>
     </row>
@@ -28718,7 +28698,7 @@
       </c>
       <c r="J561" s="7" t="inlineStr">
         <is>
-          <t>69. kvinne</t>
+          <t>69; kvinne</t>
         </is>
       </c>
     </row>
@@ -28770,7 +28750,7 @@
       </c>
       <c r="J562" s="7" t="inlineStr">
         <is>
-          <t>242. mann</t>
+          <t>242; mann</t>
         </is>
       </c>
     </row>
@@ -28822,7 +28802,7 @@
       </c>
       <c r="J563" s="7" t="inlineStr">
         <is>
-          <t>278. mann</t>
+          <t>278; mann</t>
         </is>
       </c>
     </row>
@@ -28874,7 +28854,7 @@
       </c>
       <c r="J564" s="7" t="inlineStr">
         <is>
-          <t>284. mann</t>
+          <t>284; mann</t>
         </is>
       </c>
     </row>
@@ -28926,7 +28906,7 @@
       </c>
       <c r="J565" s="7" t="inlineStr">
         <is>
-          <t>290. mann</t>
+          <t>290; mann</t>
         </is>
       </c>
     </row>
@@ -28978,7 +28958,7 @@
       </c>
       <c r="J566" s="7" t="inlineStr">
         <is>
-          <t>124. kvinne</t>
+          <t>124; kvinne</t>
         </is>
       </c>
     </row>
@@ -29030,7 +29010,7 @@
       </c>
       <c r="J567" s="7" t="inlineStr">
         <is>
-          <t>162. kvinne</t>
+          <t>162; kvinne</t>
         </is>
       </c>
     </row>
@@ -29082,7 +29062,7 @@
       </c>
       <c r="J568" s="7" t="inlineStr">
         <is>
-          <t>209. kvinne; Fartsholder</t>
+          <t>209; kvinne; Fartsholder</t>
         </is>
       </c>
     </row>
@@ -29178,7 +29158,7 @@
       </c>
       <c r="J570" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -29230,7 +29210,7 @@
       </c>
       <c r="J571" s="7" t="inlineStr">
         <is>
-          <t>3. mann</t>
+          <t>3; mann</t>
         </is>
       </c>
     </row>
@@ -29282,7 +29262,7 @@
       </c>
       <c r="J572" s="7" t="inlineStr">
         <is>
-          <t>6. mann</t>
+          <t>6; mann</t>
         </is>
       </c>
     </row>
@@ -29334,7 +29314,7 @@
       </c>
       <c r="J573" s="7" t="inlineStr">
         <is>
-          <t>7. mann</t>
+          <t>7; mann</t>
         </is>
       </c>
     </row>
@@ -29386,7 +29366,7 @@
       </c>
       <c r="J574" s="7" t="inlineStr">
         <is>
-          <t>10. mann</t>
+          <t>10; mann</t>
         </is>
       </c>
     </row>
@@ -29438,7 +29418,7 @@
       </c>
       <c r="J575" s="7" t="inlineStr">
         <is>
-          <t>14. mann</t>
+          <t>14; mann</t>
         </is>
       </c>
     </row>
@@ -29490,7 +29470,7 @@
       </c>
       <c r="J576" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -29542,7 +29522,7 @@
       </c>
       <c r="J577" s="7" t="inlineStr">
         <is>
-          <t>70. mann</t>
+          <t>70; mann</t>
         </is>
       </c>
     </row>
@@ -29594,7 +29574,7 @@
       </c>
       <c r="J578" s="7" t="inlineStr">
         <is>
-          <t>125. mann</t>
+          <t>125; mann</t>
         </is>
       </c>
     </row>
@@ -29646,7 +29626,7 @@
       </c>
       <c r="J579" s="7" t="inlineStr">
         <is>
-          <t>127. mann</t>
+          <t>127; mann</t>
         </is>
       </c>
     </row>
@@ -29698,7 +29678,7 @@
       </c>
       <c r="J580" s="7" t="inlineStr">
         <is>
-          <t>171. mann</t>
+          <t>171; mann</t>
         </is>
       </c>
     </row>
@@ -29750,7 +29730,7 @@
       </c>
       <c r="J581" s="7" t="inlineStr">
         <is>
-          <t>226. mann</t>
+          <t>226; mann</t>
         </is>
       </c>
     </row>
@@ -29802,7 +29782,7 @@
       </c>
       <c r="J582" s="7" t="inlineStr">
         <is>
-          <t>18. kvinne</t>
+          <t>18; kvinne</t>
         </is>
       </c>
     </row>
@@ -29854,7 +29834,7 @@
       </c>
       <c r="J583" s="7" t="inlineStr">
         <is>
-          <t>21. kvinne</t>
+          <t>21; kvinne</t>
         </is>
       </c>
     </row>
@@ -29906,7 +29886,7 @@
       </c>
       <c r="J584" s="7" t="inlineStr">
         <is>
-          <t>305. mann</t>
+          <t>305; mann</t>
         </is>
       </c>
     </row>
@@ -29958,7 +29938,7 @@
       </c>
       <c r="J585" s="7" t="inlineStr">
         <is>
-          <t>26. kvinne</t>
+          <t>26; kvinne</t>
         </is>
       </c>
     </row>
@@ -30010,7 +29990,7 @@
       </c>
       <c r="J586" s="7" t="inlineStr">
         <is>
-          <t>30. kvinne</t>
+          <t>30; kvinne</t>
         </is>
       </c>
     </row>
@@ -30062,7 +30042,7 @@
       </c>
       <c r="J587" s="7" t="inlineStr">
         <is>
-          <t>32. kvinne</t>
+          <t>32; kvinne</t>
         </is>
       </c>
     </row>
@@ -30114,7 +30094,7 @@
       </c>
       <c r="J588" s="7" t="inlineStr">
         <is>
-          <t>35. kvinne</t>
+          <t>35; kvinne</t>
         </is>
       </c>
     </row>
@@ -30166,7 +30146,7 @@
       </c>
       <c r="J589" s="7" t="inlineStr">
         <is>
-          <t>38. kvinne</t>
+          <t>38; kvinne</t>
         </is>
       </c>
     </row>
@@ -30218,7 +30198,7 @@
       </c>
       <c r="J590" s="7" t="inlineStr">
         <is>
-          <t>46. kvinne</t>
+          <t>46; kvinne</t>
         </is>
       </c>
     </row>
@@ -30270,7 +30250,7 @@
       </c>
       <c r="J591" s="7" t="inlineStr">
         <is>
-          <t>447. mann</t>
+          <t>447; mann</t>
         </is>
       </c>
     </row>
@@ -30322,7 +30302,7 @@
       </c>
       <c r="J592" s="7" t="inlineStr">
         <is>
-          <t>478. mann</t>
+          <t>478; mann</t>
         </is>
       </c>
     </row>
@@ -30374,7 +30354,7 @@
       </c>
       <c r="J593" s="7" t="inlineStr">
         <is>
-          <t>479. mann</t>
+          <t>479; mann</t>
         </is>
       </c>
     </row>
@@ -30426,7 +30406,7 @@
       </c>
       <c r="J594" s="7" t="inlineStr">
         <is>
-          <t>602. mann; Fartsholder</t>
+          <t>602; mann; Fartsholder</t>
         </is>
       </c>
     </row>
@@ -30474,7 +30454,7 @@
       <c r="I595" s="7" t="inlineStr"/>
       <c r="J595" s="7" t="inlineStr">
         <is>
-          <t>87. kvinne</t>
+          <t>87; kvinne</t>
         </is>
       </c>
     </row>
@@ -30526,7 +30506,7 @@
       </c>
       <c r="J596" s="7" t="inlineStr">
         <is>
-          <t>89. kvinne</t>
+          <t>89; kvinne</t>
         </is>
       </c>
     </row>
@@ -30578,7 +30558,7 @@
       </c>
       <c r="J597" s="7" t="inlineStr">
         <is>
-          <t>95. kvinne</t>
+          <t>95; kvinne</t>
         </is>
       </c>
     </row>
@@ -30630,7 +30610,7 @@
       </c>
       <c r="J598" s="7" t="inlineStr">
         <is>
-          <t>672. mann</t>
+          <t>672; mann</t>
         </is>
       </c>
     </row>
@@ -30682,7 +30662,7 @@
       </c>
       <c r="J599" s="7" t="inlineStr">
         <is>
-          <t>112. kvinne</t>
+          <t>112; kvinne</t>
         </is>
       </c>
     </row>
@@ -30734,7 +30714,7 @@
       </c>
       <c r="J600" s="7" t="inlineStr">
         <is>
-          <t>768. mann</t>
+          <t>768; mann</t>
         </is>
       </c>
     </row>
@@ -30786,7 +30766,7 @@
       </c>
       <c r="J601" s="7" t="inlineStr">
         <is>
-          <t>229. kvinne; Fartsholder</t>
+          <t>229; kvinne; Fartsholder</t>
         </is>
       </c>
     </row>
@@ -30838,7 +30818,7 @@
       </c>
       <c r="J602" s="7" t="inlineStr">
         <is>
-          <t>1017. mann</t>
+          <t>1017; mann</t>
         </is>
       </c>
     </row>
@@ -30890,7 +30870,7 @@
       </c>
       <c r="J603" s="7" t="inlineStr">
         <is>
-          <t>357. kvinne</t>
+          <t>357; kvinne</t>
         </is>
       </c>
     </row>
@@ -30942,7 +30922,7 @@
       </c>
       <c r="J604" s="7" t="inlineStr">
         <is>
-          <t>490. kvinne</t>
+          <t>490; kvinne</t>
         </is>
       </c>
     </row>
@@ -30994,7 +30974,7 @@
       </c>
       <c r="J605" s="7" t="inlineStr">
         <is>
-          <t>537. kvinne</t>
+          <t>537; kvinne</t>
         </is>
       </c>
     </row>
@@ -31046,7 +31026,7 @@
       </c>
       <c r="J606" s="7" t="inlineStr">
         <is>
-          <t>1. mann</t>
+          <t>1; mann</t>
         </is>
       </c>
     </row>
@@ -31098,7 +31078,7 @@
       </c>
       <c r="J607" s="7" t="inlineStr">
         <is>
-          <t>5. mann</t>
+          <t>5; mann</t>
         </is>
       </c>
     </row>
@@ -31150,7 +31130,7 @@
       </c>
       <c r="J608" s="7" t="inlineStr">
         <is>
-          <t>8. mann</t>
+          <t>8; mann</t>
         </is>
       </c>
     </row>
@@ -31202,7 +31182,7 @@
       </c>
       <c r="J609" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -31254,7 +31234,7 @@
       </c>
       <c r="J610" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -31306,7 +31286,7 @@
       </c>
       <c r="J611" s="7" t="inlineStr">
         <is>
-          <t>4. kvinne</t>
+          <t>4; kvinne</t>
         </is>
       </c>
     </row>
@@ -31358,7 +31338,7 @@
       </c>
       <c r="J612" s="7" t="inlineStr">
         <is>
-          <t>5. kvinne</t>
+          <t>5; kvinne</t>
         </is>
       </c>
     </row>
@@ -31410,7 +31390,7 @@
       </c>
       <c r="J613" s="7" t="inlineStr">
         <is>
-          <t>33. mann</t>
+          <t>33; mann</t>
         </is>
       </c>
     </row>
@@ -31462,7 +31442,7 @@
       </c>
       <c r="J614" s="7" t="inlineStr">
         <is>
-          <t>10. kvinne</t>
+          <t>10; kvinne</t>
         </is>
       </c>
     </row>
@@ -31514,7 +31494,7 @@
       </c>
       <c r="J615" s="7" t="inlineStr">
         <is>
-          <t>64. mann</t>
+          <t>64; mann</t>
         </is>
       </c>
     </row>
@@ -31610,7 +31590,7 @@
       </c>
       <c r="J617" s="7" t="inlineStr">
         <is>
-          <t>87. mann</t>
+          <t>87; mann</t>
         </is>
       </c>
     </row>
@@ -31662,7 +31642,7 @@
       </c>
       <c r="J618" s="7" t="inlineStr">
         <is>
-          <t>27. kvinne</t>
+          <t>27; kvinne</t>
         </is>
       </c>
     </row>
@@ -31714,7 +31694,7 @@
       </c>
       <c r="J619" s="7" t="inlineStr">
         <is>
-          <t>43. kvinne</t>
+          <t>43; kvinne</t>
         </is>
       </c>
     </row>
@@ -31766,7 +31746,7 @@
       </c>
       <c r="J620" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -31818,7 +31798,7 @@
       </c>
       <c r="J621" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -31870,7 +31850,7 @@
       </c>
       <c r="J622" s="7" t="inlineStr">
         <is>
-          <t>1. plass totalt</t>
+          <t>1; plass totalt</t>
         </is>
       </c>
     </row>
@@ -31922,7 +31902,7 @@
       </c>
       <c r="J623" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne</t>
+          <t>1; kvinne</t>
         </is>
       </c>
     </row>
@@ -31974,7 +31954,7 @@
       </c>
       <c r="J624" s="7" t="inlineStr">
         <is>
-          <t>1. plass</t>
+          <t>1; plass</t>
         </is>
       </c>
     </row>
@@ -32022,7 +32002,7 @@
       <c r="I625" s="7" t="inlineStr"/>
       <c r="J625" s="7" t="inlineStr">
         <is>
-          <t>2. kvinne</t>
+          <t>2; kvinne</t>
         </is>
       </c>
     </row>
@@ -33380,11 +33360,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="J653" s="7" t="inlineStr">
-        <is>
-          <t>SK Vidar aktiv medlem</t>
-        </is>
-      </c>
+      <c r="J653" s="7" t="inlineStr"/>
     </row>
     <row r="654">
       <c r="A654" s="6" t="inlineStr">
@@ -33432,11 +33408,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="J654" s="7" t="inlineStr">
-        <is>
-          <t>Slack workspace, svak navnematch</t>
-        </is>
-      </c>
+      <c r="J654" s="7" t="inlineStr"/>
     </row>
     <row r="655">
       <c r="A655" s="6" t="inlineStr">
@@ -33484,11 +33456,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="J655" s="7" t="inlineStr">
-        <is>
-          <t>SK Vidar aktiv medlem; Slack</t>
-        </is>
-      </c>
+      <c r="J655" s="7" t="inlineStr"/>
     </row>
     <row r="656">
       <c r="A656" s="6" t="inlineStr">
@@ -33538,7 +33506,7 @@
       </c>
       <c r="J656" s="7" t="inlineStr">
         <is>
-          <t>Offisiell Vidar; SK Vidar aktiv medlem; Slack</t>
+          <t>Offisiell Vidar</t>
         </is>
       </c>
     </row>
@@ -33590,7 +33558,7 @@
       </c>
       <c r="J657" s="7" t="inlineStr">
         <is>
-          <t>Offisiell Vidar; SK Vidar aktiv medlem; Slack</t>
+          <t>Offisiell Vidar</t>
         </is>
       </c>
     </row>
@@ -33642,7 +33610,7 @@
       </c>
       <c r="J658" s="7" t="inlineStr">
         <is>
-          <t>Offisiell Vidar; SK Vidar aktiv medlem</t>
+          <t>Offisiell Vidar</t>
         </is>
       </c>
     </row>
@@ -33692,11 +33660,7 @@
           <t>296</t>
         </is>
       </c>
-      <c r="J659" s="7" t="inlineStr">
-        <is>
-          <t>Slack workspace, svak navnematch</t>
-        </is>
-      </c>
+      <c r="J659" s="7" t="inlineStr"/>
     </row>
     <row r="660">
       <c r="A660" s="6" t="inlineStr">
@@ -33746,7 +33710,7 @@
       </c>
       <c r="J660" s="7" t="inlineStr">
         <is>
-          <t>Offisiell Vidar; SK Vidar aktiv medlem</t>
+          <t>Offisiell Vidar</t>
         </is>
       </c>
     </row>
@@ -33798,7 +33762,7 @@
       </c>
       <c r="J661" s="7" t="inlineStr">
         <is>
-          <t>Offisiell Vidar; SK Vidar aktiv medlem</t>
+          <t>Offisiell Vidar</t>
         </is>
       </c>
     </row>
@@ -33900,11 +33864,7 @@
           <t>741</t>
         </is>
       </c>
-      <c r="J663" s="7" t="inlineStr">
-        <is>
-          <t>SK Vidar aktiv medlem; Slack</t>
-        </is>
-      </c>
+      <c r="J663" s="7" t="inlineStr"/>
     </row>
     <row r="664">
       <c r="A664" s="6" t="inlineStr">
@@ -33954,7 +33914,7 @@
       </c>
       <c r="J664" s="7" t="inlineStr">
         <is>
-          <t>Offisiell Vidar; SK Vidar aktiv medlem</t>
+          <t>Offisiell Vidar</t>
         </is>
       </c>
     </row>
@@ -34056,11 +34016,7 @@
           <t>2755</t>
         </is>
       </c>
-      <c r="J666" s="7" t="inlineStr">
-        <is>
-          <t>Slack; SK Vidar fellestrening</t>
-        </is>
-      </c>
+      <c r="J666" s="7" t="inlineStr"/>
     </row>
     <row r="667">
       <c r="A667" s="6" t="inlineStr">
@@ -34110,7 +34066,7 @@
       </c>
       <c r="J667" s="7" t="inlineStr">
         <is>
-          <t>1. kvinne, 1. K30-34</t>
+          <t>1; kvinne, 1; K30-34</t>
         </is>
       </c>
     </row>
@@ -34160,11 +34116,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="J668" s="7" t="inlineStr">
-        <is>
-          <t>Relatert utøver, FIN</t>
-        </is>
-      </c>
+      <c r="J668" s="7" t="inlineStr"/>
     </row>
     <row r="669">
       <c r="A669" s="6" t="inlineStr">
@@ -34266,7 +34218,7 @@
       </c>
       <c r="J670" s="7" t="inlineStr">
         <is>
-          <t>3. M60-64</t>
+          <t>3; M60-64</t>
         </is>
       </c>
     </row>
@@ -34370,7 +34322,7 @@
       </c>
       <c r="J672" s="7" t="inlineStr">
         <is>
-          <t>95. plass menn totalt</t>
+          <t>95; plass menn totalt</t>
         </is>
       </c>
     </row>
@@ -34468,11 +34420,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="J674" s="7" t="inlineStr">
-        <is>
-          <t>SK Vidar Slack</t>
-        </is>
-      </c>
+      <c r="J674" s="7" t="inlineStr"/>
     </row>
     <row r="675">
       <c r="A675" s="6" t="inlineStr">
@@ -35238,7 +35186,7 @@
       </c>
       <c r="J689" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne</t>
+          <t>3; kvinne</t>
         </is>
       </c>
     </row>
@@ -39550,7 +39498,7 @@
       </c>
       <c r="J774" s="7" t="inlineStr">
         <is>
-          <t>trail, 2. kvinne</t>
+          <t>trail, 2; kvinne</t>
         </is>
       </c>
     </row>
@@ -51350,7 +51298,7 @@
       </c>
       <c r="J1017" s="7" t="inlineStr">
         <is>
-          <t>Klasseplass 8. M-rangering 144. BIB 281</t>
+          <t>Klasseplass 8; M-rangering 144; BIB 281</t>
         </is>
       </c>
     </row>
@@ -51690,7 +51638,7 @@
       </c>
       <c r="J1024" s="7" t="inlineStr">
         <is>
-          <t>Klassevinner. Beste kvinne totalt</t>
+          <t>Klassevinner; Beste kvinne totalt</t>
         </is>
       </c>
     </row>
@@ -51786,7 +51734,7 @@
       <c r="I1026" s="7" t="inlineStr"/>
       <c r="J1026" s="7" t="inlineStr">
         <is>
-          <t>Manuell registrering fra tekst. BIB 11436. NC</t>
+          <t>BIB 11436; NC</t>
         </is>
       </c>
     </row>
@@ -51882,7 +51830,7 @@
       </c>
       <c r="J1028" s="7" t="inlineStr">
         <is>
-          <t>BIB 21457. Guntid 2 27. Klasseplass 97. NC/klasse MSR</t>
+          <t>BIB 21457; Guntid 2 27; Klasseplass 97; NC/klasse MSR</t>
         </is>
       </c>
     </row>
@@ -51934,7 +51882,7 @@
       </c>
       <c r="J1029" s="7" t="inlineStr">
         <is>
-          <t>Offisiell resultattid 5 39. Nettotid 3 12. Guntid 5 39</t>
+          <t>Offisiell resultattid 5 39; Nettotid 3 12; Guntid 5 39</t>
         </is>
       </c>
     </row>
@@ -52466,7 +52414,7 @@
       </c>
       <c r="J1040" s="7" t="inlineStr">
         <is>
-          <t>3. plass totalt kvinner</t>
+          <t>3; plass totalt kvinner</t>
         </is>
       </c>
     </row>
@@ -59138,7 +59086,7 @@
       </c>
       <c r="J1178" s="7" t="inlineStr">
         <is>
-          <t>MSR, kat. 27</t>
+          <t>MSR, kat; 27</t>
         </is>
       </c>
     </row>
@@ -59575,14 +59523,10 @@
           <t>18:41</t>
         </is>
       </c>
-      <c r="I1187" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="I1187" s="7" t="inlineStr"/>
       <c r="J1187" s="7" t="inlineStr">
         <is>
-          <t>1. plass M14</t>
+          <t>1; plass M14</t>
         </is>
       </c>
     </row>
@@ -59627,14 +59571,10 @@
           <t>35:22</t>
         </is>
       </c>
-      <c r="I1188" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="I1188" s="7" t="inlineStr"/>
       <c r="J1188" s="7" t="inlineStr">
         <is>
-          <t>1. plass K23</t>
+          <t>1; plass K23</t>
         </is>
       </c>
     </row>
@@ -59679,14 +59619,10 @@
           <t>1:39:02</t>
         </is>
       </c>
-      <c r="I1189" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="I1189" s="7" t="inlineStr"/>
       <c r="J1189" s="7" t="inlineStr">
         <is>
-          <t>1. plass K23, para</t>
+          <t>1; plass K23, para</t>
         </is>
       </c>
     </row>
@@ -60890,7 +60826,7 @@
       <c r="I1214" s="7" t="inlineStr"/>
       <c r="J1214" s="7" t="inlineStr">
         <is>
-          <t>Ble tøft da vinden økte ved ca. 10 km, men vakker løype og god stemning</t>
+          <t>Ble tøft da vinden økte ved ca; 10 km, men vakker løype og god stemning</t>
         </is>
       </c>
     </row>
@@ -63590,7 +63526,7 @@
       </c>
       <c r="J1275" s="7" t="inlineStr">
         <is>
-          <t>4. plass</t>
+          <t>4; plass</t>
         </is>
       </c>
     </row>
@@ -66662,7 +66598,7 @@
       <c r="I1342" s="7" t="inlineStr"/>
       <c r="J1342" s="7" t="inlineStr">
         <is>
-          <t>Offensiv åpning. Det kostet krefter mot slutten, men satsingen var der</t>
+          <t>Offensiv åpning på; Det kostet krefter mot slutten, men satsingen var der</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove redundant public result notes
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -688,11 +688,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
-        <is>
-          <t>startnummer 400</t>
-        </is>
-      </c>
+      <c r="J9" s="7" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -740,11 +736,7 @@
           <t>3</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>startnummer 402</t>
-        </is>
-      </c>
+      <c r="J10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -792,11 +784,7 @@
           <t>1</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
-        <is>
-          <t>terrengløp, 1. mann, klasseplass 1, startnummer 511</t>
-        </is>
-      </c>
+      <c r="J11" s="7" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -844,11 +832,7 @@
           <t>2</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>terrengløp, 2. mann, klasseplass 2, startnummer 514</t>
-        </is>
-      </c>
+      <c r="J12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Suppler Håvard Berges Stockholm-resultat
</commit_message>
<xml_diff>
--- a/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
+++ b/data/delt_oversikt/SK Vidar Langdistanse 2026.xlsx
@@ -1669,12 +1669,12 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>3. kvinne, klasseplass 3, startnummer 790, Sk Vidar</t>
+          <t>23. plass i Senior</t>
         </is>
       </c>
     </row>

</xml_diff>